<commit_message>
Finalize D1 event-level recovery and Nature figures
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D1 Sensor health/outputs/data/D1_event_windows.xlsx
+++ b/Project 1 Data Quality Assessment/D1 Sensor health/outputs/data/D1_event_windows.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H73"/>
+  <dimension ref="A1:H90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -513,27 +513,27 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45953.125</v>
+        <v>45952.25</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>45953.625</v>
+        <v>45959.70833333334</v>
       </c>
       <c r="D3" t="n">
-        <v>13</v>
+        <v>180</v>
       </c>
       <c r="E3" t="n">
-        <v>2.669304121202174</v>
+        <v>2.151271435291634</v>
       </c>
       <c r="F3" t="n">
-        <v>2.770372721020552</v>
+        <v>2.490854942851664</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Q_step</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>1.423595848943672</v>
+        <v>1.000517494124533</v>
       </c>
     </row>
     <row r="4">
@@ -543,27 +543,27 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>45953.75</v>
+        <v>45977.16666666666</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>45962.41666666666</v>
+        <v>45977.95833333334</v>
       </c>
       <c r="D4" t="n">
-        <v>209</v>
+        <v>20</v>
       </c>
       <c r="E4" t="n">
-        <v>2.471022684808087</v>
+        <v>2.51544046636314</v>
       </c>
       <c r="F4" t="n">
-        <v>2.49986135255889</v>
+        <v>2.670916488887197</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Q_regime</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>1.121581731628728</v>
+        <v>1.00000004645339</v>
       </c>
     </row>
     <row r="5">
@@ -573,27 +573,27 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>45977.16666666666</v>
+        <v>45978.25</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>45977.75</v>
+        <v>45978.75</v>
       </c>
       <c r="D5" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E5" t="n">
-        <v>2.617931355126567</v>
+        <v>2.650685922878988</v>
       </c>
       <c r="F5" t="n">
-        <v>2.763838609289453</v>
+        <v>2.809306929822704</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_step</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>1.000074592591474</v>
+        <v>1.423595848943672</v>
       </c>
     </row>
     <row r="6">
@@ -603,27 +603,27 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>45978.25</v>
+        <v>45982.70833333334</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>45978.75</v>
+        <v>45983.125</v>
       </c>
       <c r="D6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E6" t="n">
-        <v>2.650685922878988</v>
+        <v>2.597044885183251</v>
       </c>
       <c r="F6" t="n">
-        <v>2.809306929822704</v>
+        <v>2.732865775634801</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Q_step</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>1.423595848943672</v>
+        <v>1.285374529118333</v>
       </c>
     </row>
     <row r="7">
@@ -633,19 +633,19 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>45982.70833333334</v>
+        <v>46015.29166666666</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>45983.125</v>
+        <v>46015.625</v>
       </c>
       <c r="D7" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E7" t="n">
-        <v>2.597044885183251</v>
+        <v>2.754453581023049</v>
       </c>
       <c r="F7" t="n">
-        <v>2.732865775634801</v>
+        <v>2.889382418872442</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>1.285374529118333</v>
+        <v>1.006867340116572</v>
       </c>
     </row>
     <row r="8">
@@ -663,49 +663,49 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>46015.29166666666</v>
+        <v>46031.375</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>46015.625</v>
+        <v>46031.95833333334</v>
       </c>
       <c r="D8" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E8" t="n">
-        <v>2.754453581023049</v>
+        <v>2.5</v>
       </c>
       <c r="F8" t="n">
-        <v>2.889382418872442</v>
+        <v>2.5</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_step</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>1.006867340116572</v>
+        <v>1.623688071749023</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>DO_1_2</t>
+          <t>DO_1_3</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>46029.20833333334</v>
+        <v>45952.625</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>46029.41666666666</v>
+        <v>45952.875</v>
       </c>
       <c r="D9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E9" t="n">
-        <v>2.628489943253618</v>
+        <v>2.67580637643619</v>
       </c>
       <c r="F9" t="n">
-        <v>2.737006903365002</v>
+        <v>2.733973982298676</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -713,37 +713,37 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>1.087273922427159</v>
+        <v>1.00977557542446</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>DO_1_2</t>
+          <t>DO_1_3</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>46029.54166666666</v>
+        <v>45954.95833333334</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>46029.75</v>
+        <v>45955.29166666666</v>
       </c>
       <c r="D10" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E10" t="n">
-        <v>2.56991063842729</v>
+        <v>2.5</v>
       </c>
       <c r="F10" t="n">
-        <v>2.77321471413416</v>
+        <v>2.5</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_step</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>1.281983908260925</v>
+        <v>2.541622006929802</v>
       </c>
     </row>
     <row r="11">
@@ -753,19 +753,19 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>45952.625</v>
+        <v>46029.20833333334</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>45952.875</v>
+        <v>46029.45833333334</v>
       </c>
       <c r="D11" t="n">
         <v>7</v>
       </c>
       <c r="E11" t="n">
-        <v>2.67580637643619</v>
+        <v>2.814142094241534</v>
       </c>
       <c r="F11" t="n">
-        <v>2.733973982298676</v>
+        <v>2.901820370597318</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -773,7 +773,7 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>1.00977557542446</v>
+        <v>1.048761737961288</v>
       </c>
     </row>
     <row r="12">
@@ -783,27 +783,27 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>46029.20833333334</v>
+        <v>46068.79166666666</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>46029.45833333334</v>
+        <v>46069.41666666666</v>
       </c>
       <c r="D12" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="E12" t="n">
-        <v>2.814142094241534</v>
+        <v>2.5</v>
       </c>
       <c r="F12" t="n">
-        <v>2.901820370597318</v>
+        <v>2.5</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_step</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>1.048761737961288</v>
+        <v>2.24010207548955</v>
       </c>
     </row>
     <row r="13">
@@ -1236,10 +1236,10 @@
         <v>45914.25</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>45926.70833333334</v>
+        <v>45923.20833333334</v>
       </c>
       <c r="D27" t="n">
-        <v>300</v>
+        <v>216</v>
       </c>
       <c r="E27" t="n">
         <v>2.5</v>
@@ -1263,19 +1263,19 @@
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>45943.45833333334</v>
+        <v>45932.41666666666</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>45943.66666666666</v>
+        <v>45932.625</v>
       </c>
       <c r="D28" t="n">
         <v>6</v>
       </c>
       <c r="E28" t="n">
-        <v>2.681089385898379</v>
+        <v>2.8576307760076</v>
       </c>
       <c r="F28" t="n">
-        <v>2.745318634673053</v>
+        <v>2.905041855817255</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>1.004340877014071</v>
+        <v>1.000000003707427</v>
       </c>
     </row>
     <row r="29">
@@ -1293,27 +1293,27 @@
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>45954.20833333334</v>
+        <v>45933.25</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>45954.45833333334</v>
+        <v>45933.66666666666</v>
       </c>
       <c r="D29" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E29" t="n">
-        <v>2.5</v>
+        <v>2.715725978999145</v>
       </c>
       <c r="F29" t="n">
-        <v>2.5</v>
+        <v>2.855430384698202</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Q_step</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H29" t="n">
-        <v>2.24010207548955</v>
+        <v>1.00001596166619</v>
       </c>
     </row>
     <row r="30">
@@ -1323,19 +1323,19 @@
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>46012.16666666666</v>
+        <v>45935.33333333334</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>46012.375</v>
+        <v>45935.58333333334</v>
       </c>
       <c r="D30" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E30" t="n">
-        <v>2.668447168786347</v>
+        <v>2.869900144214022</v>
       </c>
       <c r="F30" t="n">
-        <v>2.728167845843344</v>
+        <v>2.891838461848703</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1343,7 +1343,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>1.000040627835267</v>
+        <v>1.000004089993105</v>
       </c>
     </row>
     <row r="31">
@@ -1353,19 +1353,19 @@
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>46015.16666666666</v>
+        <v>45949.75</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>46015.45833333334</v>
+        <v>45949.95833333334</v>
       </c>
       <c r="D31" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E31" t="n">
-        <v>2.632442099658302</v>
+        <v>2.746670604989188</v>
       </c>
       <c r="F31" t="n">
-        <v>2.707099187084153</v>
+        <v>2.867587939799336</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>1.005069353080617</v>
+        <v>1.017767620865028</v>
       </c>
     </row>
     <row r="32">
@@ -1383,27 +1383,27 @@
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>46064.20833333334</v>
+        <v>45953.79166666666</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>46064.5</v>
+        <v>45954.66666666666</v>
       </c>
       <c r="D32" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="E32" t="n">
-        <v>2.752899050823816</v>
+        <v>2.5</v>
       </c>
       <c r="F32" t="n">
-        <v>2.849062511830852</v>
+        <v>2.5</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_step</t>
         </is>
       </c>
       <c r="H32" t="n">
-        <v>1.00016713661482</v>
+        <v>1.749799171982965</v>
       </c>
     </row>
     <row r="33">
@@ -1413,27 +1413,27 @@
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>46068.70833333334</v>
+        <v>45986.79166666666</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>46069.16666666666</v>
+        <v>45987.04166666666</v>
       </c>
       <c r="D33" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="E33" t="n">
-        <v>2.659300017482196</v>
+        <v>2.5</v>
       </c>
       <c r="F33" t="n">
-        <v>2.822869313003498</v>
+        <v>2.5</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_step</t>
         </is>
       </c>
       <c r="H33" t="n">
-        <v>1.000052489251805</v>
+        <v>2.541622006929802</v>
       </c>
     </row>
     <row r="34">
@@ -1443,27 +1443,27 @@
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>46069.45833333334</v>
+        <v>46002.875</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>46069.66666666666</v>
+        <v>46003.08333333334</v>
       </c>
       <c r="D34" t="n">
         <v>6</v>
       </c>
       <c r="E34" t="n">
-        <v>2.507016709960635</v>
+        <v>2.5</v>
       </c>
       <c r="F34" t="n">
-        <v>2.619198850158543</v>
+        <v>2.5</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_step</t>
         </is>
       </c>
       <c r="H34" t="n">
-        <v>1.000004982251552</v>
+        <v>2.866863846995475</v>
       </c>
     </row>
     <row r="35">
@@ -1473,19 +1473,19 @@
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>46070.20833333334</v>
+        <v>46012.16666666666</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>46070.625</v>
+        <v>46012.375</v>
       </c>
       <c r="D35" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E35" t="n">
-        <v>2.58809163181568</v>
+        <v>2.668447168786347</v>
       </c>
       <c r="F35" t="n">
-        <v>2.643736605693489</v>
+        <v>2.728167845843344</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -1493,7 +1493,7 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>1.001910606479826</v>
+        <v>1.000040627835267</v>
       </c>
     </row>
     <row r="36">
@@ -1503,19 +1503,19 @@
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>46072.70833333334</v>
+        <v>46064.20833333334</v>
       </c>
       <c r="C36" s="2" t="n">
-        <v>46072.91666666666</v>
+        <v>46064.5</v>
       </c>
       <c r="D36" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E36" t="n">
-        <v>2.605294710093437</v>
+        <v>2.752899050823816</v>
       </c>
       <c r="F36" t="n">
-        <v>2.684925504851897</v>
+        <v>2.849062511830852</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>1.001865330224722</v>
+        <v>1.00016713661482</v>
       </c>
     </row>
     <row r="37">
@@ -1533,19 +1533,19 @@
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>46084.375</v>
+        <v>46068.70833333334</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>46084.625</v>
+        <v>46069.16666666666</v>
       </c>
       <c r="D37" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E37" t="n">
-        <v>2.835966088247843</v>
+        <v>2.659300017482196</v>
       </c>
       <c r="F37" t="n">
-        <v>2.858030849130147</v>
+        <v>2.822869313003498</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -1553,7 +1553,7 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>1.005803109498485</v>
+        <v>1.000052489251805</v>
       </c>
     </row>
     <row r="38">
@@ -1563,19 +1563,19 @@
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>46102.83333333334</v>
+        <v>46069.45833333334</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>46103.41666666666</v>
+        <v>46069.66666666666</v>
       </c>
       <c r="D38" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="E38" t="n">
-        <v>2</v>
+        <v>2.507016709960635</v>
       </c>
       <c r="F38" t="n">
-        <v>2.188396148632055</v>
+        <v>2.619198850158543</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -1583,7 +1583,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>1.000000000467794</v>
+        <v>1.000004982251552</v>
       </c>
     </row>
     <row r="39">
@@ -1593,19 +1593,19 @@
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>46103.66666666666</v>
+        <v>46070.20833333334</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>46104.125</v>
+        <v>46070.625</v>
       </c>
       <c r="D39" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E39" t="n">
-        <v>2.497046139473277</v>
+        <v>2.58809163181568</v>
       </c>
       <c r="F39" t="n">
-        <v>2.607939938695307</v>
+        <v>2.643736605693489</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -1613,7 +1613,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>1.000000039380453</v>
+        <v>1.001910606479826</v>
       </c>
     </row>
     <row r="40">
@@ -1623,19 +1623,19 @@
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>46104.45833333334</v>
+        <v>46084.375</v>
       </c>
       <c r="C40" s="2" t="n">
-        <v>46104.875</v>
+        <v>46084.625</v>
       </c>
       <c r="D40" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>2.512394845773965</v>
+        <v>2.835966088247843</v>
       </c>
       <c r="F40" t="n">
-        <v>2.779489266082209</v>
+        <v>2.858030849130147</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -1643,7 +1643,7 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>1.09718383978607</v>
+        <v>1.005803109498485</v>
       </c>
     </row>
     <row r="41">
@@ -1653,19 +1653,19 @@
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>46109.95833333334</v>
+        <v>46102.83333333334</v>
       </c>
       <c r="C41" s="2" t="n">
-        <v>46110.20833333334</v>
+        <v>46103.41666666666</v>
       </c>
       <c r="D41" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="E41" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="F41" t="n">
-        <v>2.558879692815726</v>
+        <v>2.188396148632055</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
@@ -1673,29 +1673,29 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>1.586270319473582</v>
+        <v>1.000000000467794</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>DO_2_4</t>
+          <t>DO_2_3</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>45909.70833333334</v>
+        <v>46103.66666666666</v>
       </c>
       <c r="C42" s="2" t="n">
-        <v>45909.91666666666</v>
+        <v>46104.125</v>
       </c>
       <c r="D42" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E42" t="n">
-        <v>2.70713776458959</v>
+        <v>2.497046139473277</v>
       </c>
       <c r="F42" t="n">
-        <v>2.771030551549705</v>
+        <v>2.607939938695307</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -1703,29 +1703,29 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>1.021064670664183</v>
+        <v>1.000000039380453</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>DO_2_4</t>
+          <t>DO_2_3</t>
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>45920.5</v>
+        <v>46104.45833333334</v>
       </c>
       <c r="C43" s="2" t="n">
-        <v>45921.04166666666</v>
+        <v>46104.875</v>
       </c>
       <c r="D43" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E43" t="n">
-        <v>2.584449116056976</v>
+        <v>2.512394845773965</v>
       </c>
       <c r="F43" t="n">
-        <v>2.734954268322661</v>
+        <v>2.779489266082209</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -1733,29 +1733,29 @@
         </is>
       </c>
       <c r="H43" t="n">
-        <v>1.000654868107215</v>
+        <v>1.09718383978607</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>DO_2_4</t>
+          <t>DO_2_3</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>45952</v>
+        <v>46109.95833333334</v>
       </c>
       <c r="C44" s="2" t="n">
-        <v>45952.29166666666</v>
+        <v>46110.20833333334</v>
       </c>
       <c r="D44" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>2.617381158835892</v>
+        <v>2.5</v>
       </c>
       <c r="F44" t="n">
-        <v>2.748156902964956</v>
+        <v>2.558879692815726</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -1763,7 +1763,7 @@
         </is>
       </c>
       <c r="H44" t="n">
-        <v>1.002373070803649</v>
+        <v>1.586270319473582</v>
       </c>
     </row>
     <row r="45">
@@ -1773,19 +1773,19 @@
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>45982.66666666666</v>
+        <v>45909.70833333334</v>
       </c>
       <c r="C45" s="2" t="n">
-        <v>45983.54166666666</v>
+        <v>45909.91666666666</v>
       </c>
       <c r="D45" t="n">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="E45" t="n">
-        <v>2.545105371609574</v>
+        <v>2.70713776458959</v>
       </c>
       <c r="F45" t="n">
-        <v>2.676906611498591</v>
+        <v>2.771030551549705</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -1793,7 +1793,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>1.0000017189618</v>
+        <v>1.021064670664183</v>
       </c>
     </row>
     <row r="46">
@@ -1803,27 +1803,27 @@
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>45984.91666666666</v>
+        <v>45920.5</v>
       </c>
       <c r="C46" s="2" t="n">
-        <v>45985.58333333334</v>
+        <v>45921.04166666666</v>
       </c>
       <c r="D46" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E46" t="n">
-        <v>2.5</v>
+        <v>2.584449116056976</v>
       </c>
       <c r="F46" t="n">
-        <v>2.733102015436797</v>
+        <v>2.734954268322661</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Q_step</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H46" t="n">
-        <v>1.229296703595475</v>
+        <v>1.000654868107215</v>
       </c>
     </row>
     <row r="47">
@@ -1833,27 +1833,27 @@
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>45998.625</v>
+        <v>45952</v>
       </c>
       <c r="C47" s="2" t="n">
-        <v>45998.875</v>
+        <v>45952.29166666666</v>
       </c>
       <c r="D47" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E47" t="n">
-        <v>2.543637438319223</v>
+        <v>2.617381158835892</v>
       </c>
       <c r="F47" t="n">
-        <v>2.744699115030357</v>
+        <v>2.748156902964956</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Q_step</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H47" t="n">
-        <v>1.623688071749023</v>
+        <v>1.002373070803649</v>
       </c>
     </row>
     <row r="48">
@@ -1863,19 +1863,19 @@
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>46011.5</v>
+        <v>45982.66666666666</v>
       </c>
       <c r="C48" s="2" t="n">
-        <v>46011.83333333334</v>
+        <v>45983.54166666666</v>
       </c>
       <c r="D48" t="n">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="E48" t="n">
-        <v>2.442125375774663</v>
+        <v>2.545105371609574</v>
       </c>
       <c r="F48" t="n">
-        <v>2.50729738658907</v>
+        <v>2.676906611498591</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -1883,7 +1883,7 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>1.00000001027265</v>
+        <v>1.0000017189618</v>
       </c>
     </row>
     <row r="49">
@@ -1893,27 +1893,27 @@
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>46011.91666666666</v>
+        <v>45984.91666666666</v>
       </c>
       <c r="C49" s="2" t="n">
-        <v>46012.16666666666</v>
+        <v>45986.33333333334</v>
       </c>
       <c r="D49" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="E49" t="n">
-        <v>2.326615776323986</v>
+        <v>2.5</v>
       </c>
       <c r="F49" t="n">
-        <v>2.405759655450241</v>
+        <v>2.613220978926444</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_step</t>
         </is>
       </c>
       <c r="H49" t="n">
-        <v>1.000022140595145</v>
+        <v>1.229296703595475</v>
       </c>
     </row>
     <row r="50">
@@ -1923,27 +1923,27 @@
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>46013.5</v>
+        <v>45998.625</v>
       </c>
       <c r="C50" s="2" t="n">
-        <v>46014.16666666666</v>
+        <v>45998.875</v>
       </c>
       <c r="D50" t="n">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="E50" t="n">
-        <v>2.344867546996693</v>
+        <v>2.543637438319223</v>
       </c>
       <c r="F50" t="n">
-        <v>2.592431403304887</v>
+        <v>2.744699115030357</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_step</t>
         </is>
       </c>
       <c r="H50" t="n">
-        <v>1.000000012974778</v>
+        <v>1.623688071749023</v>
       </c>
     </row>
     <row r="51">
@@ -1953,27 +1953,27 @@
         </is>
       </c>
       <c r="B51" s="2" t="n">
-        <v>46029.66666666666</v>
+        <v>46000.625</v>
       </c>
       <c r="C51" s="2" t="n">
-        <v>46029.875</v>
+        <v>46001.04166666666</v>
       </c>
       <c r="D51" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E51" t="n">
-        <v>2.365933985321182</v>
+        <v>2.5</v>
       </c>
       <c r="F51" t="n">
-        <v>2.558276279862052</v>
+        <v>2.5</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_step</t>
         </is>
       </c>
       <c r="H51" t="n">
-        <v>1.001473515745823</v>
+        <v>2.541622006929802</v>
       </c>
     </row>
     <row r="52">
@@ -1983,19 +1983,19 @@
         </is>
       </c>
       <c r="B52" s="2" t="n">
-        <v>46096.66666666666</v>
+        <v>46011.5</v>
       </c>
       <c r="C52" s="2" t="n">
-        <v>46097</v>
+        <v>46011.83333333334</v>
       </c>
       <c r="D52" t="n">
         <v>9</v>
       </c>
       <c r="E52" t="n">
-        <v>2.747872100931619</v>
+        <v>2.442125375774663</v>
       </c>
       <c r="F52" t="n">
-        <v>2.836444563671351</v>
+        <v>2.50729738658907</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -2003,7 +2003,7 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>1.022509901506786</v>
+        <v>1.00000001027265</v>
       </c>
     </row>
     <row r="53">
@@ -2013,19 +2013,19 @@
         </is>
       </c>
       <c r="B53" s="2" t="n">
-        <v>46102.875</v>
+        <v>46011.91666666666</v>
       </c>
       <c r="C53" s="2" t="n">
-        <v>46103.33333333334</v>
+        <v>46012.16666666666</v>
       </c>
       <c r="D53" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="E53" t="n">
-        <v>2</v>
+        <v>2.326615776323986</v>
       </c>
       <c r="F53" t="n">
-        <v>2.125412860902796</v>
+        <v>2.405759655450241</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -2033,7 +2033,7 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>1.017645950689936</v>
+        <v>1.000022140595145</v>
       </c>
     </row>
     <row r="54">
@@ -2043,19 +2043,19 @@
         </is>
       </c>
       <c r="B54" s="2" t="n">
-        <v>46103.70833333334</v>
+        <v>46013.5</v>
       </c>
       <c r="C54" s="2" t="n">
-        <v>46104.08333333334</v>
+        <v>46014.16666666666</v>
       </c>
       <c r="D54" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="E54" t="n">
-        <v>2.5913563273228</v>
+        <v>2.344867546996693</v>
       </c>
       <c r="F54" t="n">
-        <v>2.719381848821334</v>
+        <v>2.592431403304887</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -2063,59 +2063,59 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>1.008731230377252</v>
+        <v>1.000000012974778</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>ORP_1_2</t>
+          <t>DO_2_4</t>
         </is>
       </c>
       <c r="B55" s="2" t="n">
-        <v>46011.91666666666</v>
+        <v>46014.33333333334</v>
       </c>
       <c r="C55" s="2" t="n">
-        <v>46012.125</v>
+        <v>46014.70833333334</v>
       </c>
       <c r="D55" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>2.737078226139449</v>
+        <v>2.727395929484985</v>
       </c>
       <c r="F55" t="n">
-        <v>2.847472325151764</v>
+        <v>2.807299739265898</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_step</t>
         </is>
       </c>
       <c r="H55" t="n">
-        <v>1.000313907608093</v>
+        <v>1.423595848943672</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>ORP_1_2</t>
+          <t>DO_2_4</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
-        <v>46017.375</v>
+        <v>46096.66666666666</v>
       </c>
       <c r="C56" s="2" t="n">
-        <v>46017.83333333334</v>
+        <v>46097</v>
       </c>
       <c r="D56" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E56" t="n">
-        <v>2.167772005843953</v>
+        <v>2.747872100931619</v>
       </c>
       <c r="F56" t="n">
-        <v>2.597986119624171</v>
+        <v>2.836444563671351</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
@@ -2123,59 +2123,59 @@
         </is>
       </c>
       <c r="H56" t="n">
-        <v>1.000380090649229</v>
+        <v>1.022509901506786</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ORP_1_2</t>
+          <t>DO_2_4</t>
         </is>
       </c>
       <c r="B57" s="2" t="n">
-        <v>46018</v>
+        <v>46102.875</v>
       </c>
       <c r="C57" s="2" t="n">
-        <v>46038.25</v>
+        <v>46103.33333333334</v>
       </c>
       <c r="D57" t="n">
-        <v>487</v>
+        <v>12</v>
       </c>
       <c r="E57" t="n">
-        <v>2.317959986394953</v>
+        <v>2</v>
       </c>
       <c r="F57" t="n">
-        <v>2.497788572677653</v>
+        <v>2.125412860902796</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Q_regime</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H57" t="n">
-        <v>1.081134041730266</v>
+        <v>1.017645950689936</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ORP_1_2</t>
+          <t>DO_2_4</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
-        <v>46063.875</v>
+        <v>46103.70833333334</v>
       </c>
       <c r="C58" s="2" t="n">
-        <v>46064.08333333334</v>
+        <v>46104.08333333334</v>
       </c>
       <c r="D58" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>2.46371245656945</v>
+        <v>2.5913563273228</v>
       </c>
       <c r="F58" t="n">
-        <v>2.641043884053045</v>
+        <v>2.719381848821334</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -2183,7 +2183,7 @@
         </is>
       </c>
       <c r="H58" t="n">
-        <v>1.010767658751164</v>
+        <v>1.008731230377252</v>
       </c>
     </row>
     <row r="59">
@@ -2193,19 +2193,19 @@
         </is>
       </c>
       <c r="B59" s="2" t="n">
-        <v>46066</v>
+        <v>46011.91666666666</v>
       </c>
       <c r="C59" s="2" t="n">
-        <v>46066.25</v>
+        <v>46012.125</v>
       </c>
       <c r="D59" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E59" t="n">
-        <v>2.317494233342275</v>
+        <v>2.737078226139449</v>
       </c>
       <c r="F59" t="n">
-        <v>2.505182217827872</v>
+        <v>2.847472325151764</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -2213,7 +2213,7 @@
         </is>
       </c>
       <c r="H59" t="n">
-        <v>1.038916563232165</v>
+        <v>1.000313907608093</v>
       </c>
     </row>
     <row r="60">
@@ -2223,19 +2223,19 @@
         </is>
       </c>
       <c r="B60" s="2" t="n">
-        <v>46067.33333333334</v>
+        <v>46017.375</v>
       </c>
       <c r="C60" s="2" t="n">
-        <v>46067.54166666666</v>
+        <v>46017.83333333334</v>
       </c>
       <c r="D60" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E60" t="n">
-        <v>2.651713442492882</v>
+        <v>2.167772005843953</v>
       </c>
       <c r="F60" t="n">
-        <v>2.772109368538855</v>
+        <v>2.597986119624171</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -2243,7 +2243,7 @@
         </is>
       </c>
       <c r="H60" t="n">
-        <v>1.056283906171612</v>
+        <v>1.000380090649229</v>
       </c>
     </row>
     <row r="61">
@@ -2253,259 +2253,259 @@
         </is>
       </c>
       <c r="B61" s="2" t="n">
-        <v>46069.75</v>
+        <v>46018</v>
       </c>
       <c r="C61" s="2" t="n">
-        <v>46125.70833333334</v>
+        <v>46025.20833333334</v>
       </c>
       <c r="D61" t="n">
-        <v>1344</v>
+        <v>174</v>
       </c>
       <c r="E61" t="n">
-        <v>2.214576517713109</v>
+        <v>2.317959986394953</v>
       </c>
       <c r="F61" t="n">
-        <v>2.496270564148117</v>
+        <v>2.492738182474997</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_regime</t>
         </is>
       </c>
       <c r="H61" t="n">
-        <v>1.00058020526325</v>
+        <v>1.081134041730266</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ORP_1_3</t>
+          <t>ORP_1_2</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
-        <v>45912.20833333334</v>
+        <v>46025.5</v>
       </c>
       <c r="C62" s="2" t="n">
-        <v>45912.41666666666</v>
+        <v>46027.5</v>
       </c>
       <c r="D62" t="n">
-        <v>6</v>
+        <v>49</v>
       </c>
       <c r="E62" t="n">
-        <v>2.838808585782044</v>
+        <v>2.5</v>
       </c>
       <c r="F62" t="n">
-        <v>2.916402563418345</v>
+        <v>2.5</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Q_step</t>
+          <t>Q_regime</t>
         </is>
       </c>
       <c r="H62" t="n">
-        <v>1.51542430420249</v>
+        <v>1.803702671774002</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>ORP_1_3</t>
+          <t>ORP_1_2</t>
         </is>
       </c>
       <c r="B63" s="2" t="n">
-        <v>45944.45833333334</v>
+        <v>46030.20833333334</v>
       </c>
       <c r="C63" s="2" t="n">
-        <v>45944.70833333334</v>
+        <v>46031.95833333334</v>
       </c>
       <c r="D63" t="n">
-        <v>7</v>
+        <v>43</v>
       </c>
       <c r="E63" t="n">
-        <v>2.681541950564857</v>
+        <v>2.149987352699235</v>
       </c>
       <c r="F63" t="n">
-        <v>2.782221389952219</v>
+        <v>2.3922480432891</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Q_step</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H63" t="n">
-        <v>1.282329482970322</v>
+        <v>1.000207179248728</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>ORP_1_3</t>
+          <t>ORP_1_2</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
-        <v>45945.25</v>
+        <v>46032.41666666666</v>
       </c>
       <c r="C64" s="2" t="n">
-        <v>45945.45833333334</v>
+        <v>46032.625</v>
       </c>
       <c r="D64" t="n">
         <v>6</v>
       </c>
       <c r="E64" t="n">
-        <v>2.5</v>
+        <v>2.256477025195484</v>
       </c>
       <c r="F64" t="n">
-        <v>2.5</v>
+        <v>2.321600742859642</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Q_regime</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H64" t="n">
-        <v>1.961678843667339</v>
+        <v>1.088169856401719</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>ORP_1_3</t>
+          <t>ORP_1_2</t>
         </is>
       </c>
       <c r="B65" s="2" t="n">
-        <v>45945.79166666666</v>
+        <v>46033.625</v>
       </c>
       <c r="C65" s="2" t="n">
-        <v>45946.20833333334</v>
+        <v>46038.25</v>
       </c>
       <c r="D65" t="n">
-        <v>11</v>
+        <v>112</v>
       </c>
       <c r="E65" t="n">
-        <v>2.635659596744977</v>
+        <v>2.352648455999176</v>
       </c>
       <c r="F65" t="n">
-        <v>2.812160783667882</v>
+        <v>2.505656680806336</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Q_step</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H65" t="n">
-        <v>2.058379058668964</v>
+        <v>1.10286685173526</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>ORP_1_3</t>
+          <t>ORP_1_2</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
-        <v>45946.75</v>
+        <v>46063.875</v>
       </c>
       <c r="C66" s="2" t="n">
-        <v>45951.5</v>
+        <v>46064.08333333334</v>
       </c>
       <c r="D66" t="n">
-        <v>115</v>
+        <v>6</v>
       </c>
       <c r="E66" t="n">
-        <v>2.5</v>
+        <v>2.46371245656945</v>
       </c>
       <c r="F66" t="n">
-        <v>2.5</v>
+        <v>2.641043884053045</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Q_step</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H66" t="n">
-        <v>2.058379058668964</v>
+        <v>1.010767658751164</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>ORP_1_3</t>
+          <t>ORP_1_2</t>
         </is>
       </c>
       <c r="B67" s="2" t="n">
-        <v>45985.79166666666</v>
+        <v>46066</v>
       </c>
       <c r="C67" s="2" t="n">
-        <v>45986.125</v>
+        <v>46066.25</v>
       </c>
       <c r="D67" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E67" t="n">
-        <v>2.564243254468536</v>
+        <v>2.317494233342275</v>
       </c>
       <c r="F67" t="n">
-        <v>2.759940853427584</v>
+        <v>2.505182217827872</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Q_step</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H67" t="n">
-        <v>1.229296703595475</v>
+        <v>1.038916563232165</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>ORP_1_3</t>
+          <t>ORP_1_2</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
-        <v>46014.45833333334</v>
+        <v>46067.33333333334</v>
       </c>
       <c r="C68" s="2" t="n">
-        <v>46014.75</v>
+        <v>46067.54166666666</v>
       </c>
       <c r="D68" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E68" t="n">
-        <v>2.838559067395091</v>
+        <v>2.651713442492882</v>
       </c>
       <c r="F68" t="n">
-        <v>2.919989230357585</v>
+        <v>2.772109368538855</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Q_step</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H68" t="n">
-        <v>1.51542430420249</v>
+        <v>1.056283906171612</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>ORP_2_1</t>
+          <t>ORP_1_2</t>
         </is>
       </c>
       <c r="B69" s="2" t="n">
-        <v>45912.625</v>
+        <v>46069.75</v>
       </c>
       <c r="C69" s="2" t="n">
-        <v>45912.83333333334</v>
+        <v>46077.91666666666</v>
       </c>
       <c r="D69" t="n">
-        <v>6</v>
+        <v>197</v>
       </c>
       <c r="E69" t="n">
-        <v>2.758076189060307</v>
+        <v>2.214576517713109</v>
       </c>
       <c r="F69" t="n">
-        <v>2.80686385338087</v>
+        <v>2.475508943690873</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
@@ -2513,29 +2513,29 @@
         </is>
       </c>
       <c r="H69" t="n">
-        <v>1.00539930261449</v>
+        <v>1.00058020526325</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ORP_2_1</t>
+          <t>ORP_1_2</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
-        <v>46014.41666666666</v>
+        <v>46078.375</v>
       </c>
       <c r="C70" s="2" t="n">
-        <v>46014.66666666666</v>
+        <v>46082.125</v>
       </c>
       <c r="D70" t="n">
-        <v>7</v>
+        <v>91</v>
       </c>
       <c r="E70" t="n">
-        <v>2.741435296101974</v>
+        <v>2.5</v>
       </c>
       <c r="F70" t="n">
-        <v>2.849723924600531</v>
+        <v>2.505172739827216</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
@@ -2543,96 +2543,606 @@
         </is>
       </c>
       <c r="H70" t="n">
-        <v>1.180759797519993</v>
+        <v>1.06850037421141</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>ORP_2_1</t>
+          <t>ORP_1_2</t>
         </is>
       </c>
       <c r="B71" s="2" t="n">
-        <v>46083.5</v>
+        <v>46082.25</v>
       </c>
       <c r="C71" s="2" t="n">
-        <v>46083.75</v>
+        <v>46088.45833333334</v>
       </c>
       <c r="D71" t="n">
-        <v>7</v>
+        <v>150</v>
       </c>
       <c r="E71" t="n">
-        <v>2.469548897143255</v>
+        <v>2.370479410035172</v>
       </c>
       <c r="F71" t="n">
-        <v>2.675205925395538</v>
+        <v>2.498346242527374</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_regime</t>
         </is>
       </c>
       <c r="H71" t="n">
-        <v>1.09003124068793</v>
+        <v>1.333577532071762</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>ORP_2_2</t>
+          <t>ORP_1_2</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
-        <v>46036.75</v>
+        <v>46115</v>
       </c>
       <c r="C72" s="2" t="n">
-        <v>46037.45833333334</v>
+        <v>46115.29166666666</v>
       </c>
       <c r="D72" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="E72" t="n">
-        <v>2.5</v>
+        <v>2.356657639501725</v>
       </c>
       <c r="F72" t="n">
-        <v>2.5</v>
+        <v>2.524522307136362</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Q_regime</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H72" t="n">
-        <v>1.922445730625928</v>
+        <v>1.102732526289897</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
+          <t>ORP_1_2</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="n">
+        <v>46117.58333333334</v>
+      </c>
+      <c r="C73" s="2" t="n">
+        <v>46117.95833333334</v>
+      </c>
+      <c r="D73" t="n">
+        <v>10</v>
+      </c>
+      <c r="E73" t="n">
+        <v>2.470676739429889</v>
+      </c>
+      <c r="F73" t="n">
+        <v>2.546554579478316</v>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Q_drift</t>
+        </is>
+      </c>
+      <c r="H73" t="n">
+        <v>1.570574173197559</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>ORP_1_2</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="n">
+        <v>46118.41666666666</v>
+      </c>
+      <c r="C74" s="2" t="n">
+        <v>46122.45833333334</v>
+      </c>
+      <c r="D74" t="n">
+        <v>98</v>
+      </c>
+      <c r="E74" t="n">
+        <v>2.338714230036328</v>
+      </c>
+      <c r="F74" t="n">
+        <v>2.505987799864467</v>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Q_drift</t>
+        </is>
+      </c>
+      <c r="H74" t="n">
+        <v>1.04046058341234</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>ORP_1_3</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="n">
+        <v>45912.16666666666</v>
+      </c>
+      <c r="C75" s="2" t="n">
+        <v>45912.41666666666</v>
+      </c>
+      <c r="D75" t="n">
+        <v>7</v>
+      </c>
+      <c r="E75" t="n">
+        <v>2.81451481117033</v>
+      </c>
+      <c r="F75" t="n">
+        <v>2.878204171198647</v>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Q_step</t>
+        </is>
+      </c>
+      <c r="H75" t="n">
+        <v>1.51542430420249</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>ORP_1_3</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="n">
+        <v>45940.54166666666</v>
+      </c>
+      <c r="C76" s="2" t="n">
+        <v>45941.25</v>
+      </c>
+      <c r="D76" t="n">
+        <v>18</v>
+      </c>
+      <c r="E76" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F76" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Q_step</t>
+        </is>
+      </c>
+      <c r="H76" t="n">
+        <v>2.437776348413636</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>ORP_1_3</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="n">
+        <v>45944.25</v>
+      </c>
+      <c r="C77" s="2" t="n">
+        <v>45944.79166666666</v>
+      </c>
+      <c r="D77" t="n">
+        <v>14</v>
+      </c>
+      <c r="E77" t="n">
+        <v>2.378602582433596</v>
+      </c>
+      <c r="F77" t="n">
+        <v>2.65933923989452</v>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Q_step</t>
+        </is>
+      </c>
+      <c r="H77" t="n">
+        <v>1.282329482970322</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>ORP_1_3</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="n">
+        <v>45945.08333333334</v>
+      </c>
+      <c r="C78" s="2" t="n">
+        <v>45945.45833333334</v>
+      </c>
+      <c r="D78" t="n">
+        <v>10</v>
+      </c>
+      <c r="E78" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F78" t="n">
+        <v>2.644339225428953</v>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Q_regime</t>
+        </is>
+      </c>
+      <c r="H78" t="n">
+        <v>1.961678843667339</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>ORP_1_3</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="n">
+        <v>45945.79166666666</v>
+      </c>
+      <c r="C79" s="2" t="n">
+        <v>45946.20833333334</v>
+      </c>
+      <c r="D79" t="n">
+        <v>11</v>
+      </c>
+      <c r="E79" t="n">
+        <v>2.635659596744977</v>
+      </c>
+      <c r="F79" t="n">
+        <v>2.812160783667882</v>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Q_step</t>
+        </is>
+      </c>
+      <c r="H79" t="n">
+        <v>2.058379058668964</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>ORP_1_3</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="n">
+        <v>45946.33333333334</v>
+      </c>
+      <c r="C80" s="2" t="n">
+        <v>45948.375</v>
+      </c>
+      <c r="D80" t="n">
+        <v>50</v>
+      </c>
+      <c r="E80" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F80" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Q_regime</t>
+        </is>
+      </c>
+      <c r="H80" t="n">
+        <v>2.108098132368428</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>ORP_1_3</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="n">
+        <v>45948.875</v>
+      </c>
+      <c r="C81" s="2" t="n">
+        <v>45949.83333333334</v>
+      </c>
+      <c r="D81" t="n">
+        <v>24</v>
+      </c>
+      <c r="E81" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F81" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Q_step</t>
+        </is>
+      </c>
+      <c r="H81" t="n">
+        <v>2.648143459082469</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>ORP_1_3</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="n">
+        <v>45985.79166666666</v>
+      </c>
+      <c r="C82" s="2" t="n">
+        <v>45986.125</v>
+      </c>
+      <c r="D82" t="n">
+        <v>9</v>
+      </c>
+      <c r="E82" t="n">
+        <v>2.564243254468536</v>
+      </c>
+      <c r="F82" t="n">
+        <v>2.759940853427584</v>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Q_step</t>
+        </is>
+      </c>
+      <c r="H82" t="n">
+        <v>1.229296703595475</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>ORP_1_3</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="n">
+        <v>45986.66666666666</v>
+      </c>
+      <c r="C83" s="2" t="n">
+        <v>45987.08333333334</v>
+      </c>
+      <c r="D83" t="n">
+        <v>11</v>
+      </c>
+      <c r="E83" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F83" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Q_step</t>
+        </is>
+      </c>
+      <c r="H83" t="n">
+        <v>2.541622006929802</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>ORP_1_3</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="n">
+        <v>46014.45833333334</v>
+      </c>
+      <c r="C84" s="2" t="n">
+        <v>46014.75</v>
+      </c>
+      <c r="D84" t="n">
+        <v>8</v>
+      </c>
+      <c r="E84" t="n">
+        <v>2.838559067395091</v>
+      </c>
+      <c r="F84" t="n">
+        <v>2.919989230357585</v>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Q_step</t>
+        </is>
+      </c>
+      <c r="H84" t="n">
+        <v>1.51542430420249</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>ORP_2_1</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="n">
+        <v>45912.625</v>
+      </c>
+      <c r="C85" s="2" t="n">
+        <v>45912.83333333334</v>
+      </c>
+      <c r="D85" t="n">
+        <v>6</v>
+      </c>
+      <c r="E85" t="n">
+        <v>2.758076189060307</v>
+      </c>
+      <c r="F85" t="n">
+        <v>2.80686385338087</v>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Q_drift</t>
+        </is>
+      </c>
+      <c r="H85" t="n">
+        <v>1.00539930261449</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>ORP_2_1</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="n">
+        <v>46014.41666666666</v>
+      </c>
+      <c r="C86" s="2" t="n">
+        <v>46014.66666666666</v>
+      </c>
+      <c r="D86" t="n">
+        <v>7</v>
+      </c>
+      <c r="E86" t="n">
+        <v>2.741435296101974</v>
+      </c>
+      <c r="F86" t="n">
+        <v>2.849723924600531</v>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Q_drift</t>
+        </is>
+      </c>
+      <c r="H86" t="n">
+        <v>1.180759797519993</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>ORP_2_1</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="n">
+        <v>46083.5</v>
+      </c>
+      <c r="C87" s="2" t="n">
+        <v>46083.75</v>
+      </c>
+      <c r="D87" t="n">
+        <v>7</v>
+      </c>
+      <c r="E87" t="n">
+        <v>2.469548897143255</v>
+      </c>
+      <c r="F87" t="n">
+        <v>2.675205925395538</v>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Q_drift</t>
+        </is>
+      </c>
+      <c r="H87" t="n">
+        <v>1.09003124068793</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
           <t>ORP_2_2</t>
         </is>
       </c>
-      <c r="B73" s="2" t="n">
+      <c r="B88" s="2" t="n">
+        <v>46036.75</v>
+      </c>
+      <c r="C88" s="2" t="n">
+        <v>46037.45833333334</v>
+      </c>
+      <c r="D88" t="n">
+        <v>18</v>
+      </c>
+      <c r="E88" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F88" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Q_regime</t>
+        </is>
+      </c>
+      <c r="H88" t="n">
+        <v>1.922445730625928</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>ORP_2_2</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="n">
+        <v>46070.33333333334</v>
+      </c>
+      <c r="C89" s="2" t="n">
+        <v>46070.75</v>
+      </c>
+      <c r="D89" t="n">
+        <v>11</v>
+      </c>
+      <c r="E89" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F89" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Q_step</t>
+        </is>
+      </c>
+      <c r="H89" t="n">
+        <v>2.866863846995475</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>ORP_2_2</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="n">
         <v>46119</v>
       </c>
-      <c r="C73" s="2" t="n">
-        <v>46125.70833333334</v>
-      </c>
-      <c r="D73" t="n">
-        <v>162</v>
-      </c>
-      <c r="E73" t="n">
+      <c r="C90" s="2" t="n">
+        <v>46122.45833333334</v>
+      </c>
+      <c r="D90" t="n">
+        <v>84</v>
+      </c>
+      <c r="E90" t="n">
         <v>2.416818111700139</v>
       </c>
-      <c r="F73" t="n">
-        <v>2.499486531553705</v>
-      </c>
-      <c r="G73" t="inlineStr">
+      <c r="F90" t="n">
+        <v>2.499009739425002</v>
+      </c>
+      <c r="G90" t="inlineStr">
         <is>
           <t>Q_regime</t>
         </is>
       </c>
-      <c r="H73" t="n">
+      <c r="H90" t="n">
         <v>1.160462951377068</v>
       </c>
     </row>
@@ -2647,7 +3157,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H63"/>
+  <dimension ref="A1:H70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2729,27 +3239,27 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45953.75</v>
+        <v>45952.25</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>45962.41666666666</v>
+        <v>45959.70833333334</v>
       </c>
       <c r="D3" t="n">
-        <v>209</v>
+        <v>180</v>
       </c>
       <c r="E3" t="n">
-        <v>2.471022684808087</v>
+        <v>2.151271435291634</v>
       </c>
       <c r="F3" t="n">
-        <v>2.49986135255889</v>
+        <v>2.490854942851664</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Q_regime</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>1.121581731628728</v>
+        <v>1.000517494124533</v>
       </c>
     </row>
     <row r="4">
@@ -2759,27 +3269,27 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>46029.54166666666</v>
+        <v>46031.375</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>46029.75</v>
+        <v>46031.95833333334</v>
       </c>
       <c r="D4" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E4" t="n">
-        <v>2.56991063842729</v>
+        <v>2.5</v>
       </c>
       <c r="F4" t="n">
-        <v>2.77321471413416</v>
+        <v>2.5</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_step</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>1.281983908260925</v>
+        <v>1.623688071749023</v>
       </c>
     </row>
     <row r="5">
@@ -2789,19 +3299,19 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>45982.70833333334</v>
+        <v>45977.16666666666</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>45983.125</v>
+        <v>45977.95833333334</v>
       </c>
       <c r="D5" t="n">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="E5" t="n">
-        <v>2.597044885183251</v>
+        <v>2.51544046636314</v>
       </c>
       <c r="F5" t="n">
-        <v>2.732865775634801</v>
+        <v>2.670916488887197</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -2809,7 +3319,7 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>1.285374529118333</v>
+        <v>1.00000004645339</v>
       </c>
     </row>
     <row r="6">
@@ -2819,19 +3329,19 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>45977.16666666666</v>
+        <v>45982.70833333334</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>45977.75</v>
+        <v>45983.125</v>
       </c>
       <c r="D6" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E6" t="n">
-        <v>2.617931355126567</v>
+        <v>2.597044885183251</v>
       </c>
       <c r="F6" t="n">
-        <v>2.763838609289453</v>
+        <v>2.732865775634801</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -2839,7 +3349,7 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>1.000074592591474</v>
+        <v>1.285374529118333</v>
       </c>
     </row>
     <row r="7">
@@ -2849,27 +3359,27 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>46029.20833333334</v>
+        <v>45978.25</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>46029.41666666666</v>
+        <v>45978.75</v>
       </c>
       <c r="D7" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="E7" t="n">
-        <v>2.628489943253618</v>
+        <v>2.650685922878988</v>
       </c>
       <c r="F7" t="n">
-        <v>2.737006903365002</v>
+        <v>2.809306929822704</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_step</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>1.087273922427159</v>
+        <v>1.423595848943672</v>
       </c>
     </row>
     <row r="8">
@@ -2879,49 +3389,49 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>45978.25</v>
+        <v>46015.29166666666</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>45978.75</v>
+        <v>46015.625</v>
       </c>
       <c r="D8" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E8" t="n">
-        <v>2.650685922878988</v>
+        <v>2.754453581023049</v>
       </c>
       <c r="F8" t="n">
-        <v>2.809306929822704</v>
+        <v>2.889382418872442</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Q_step</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>1.423595848943672</v>
+        <v>1.006867340116572</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>DO_1_2</t>
+          <t>DO_1_3</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>45953.125</v>
+        <v>45954.95833333334</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>45953.625</v>
+        <v>45955.29166666666</v>
       </c>
       <c r="D9" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E9" t="n">
-        <v>2.669304121202174</v>
+        <v>2.5</v>
       </c>
       <c r="F9" t="n">
-        <v>2.770372721020552</v>
+        <v>2.5</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -2929,37 +3439,37 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>1.423595848943672</v>
+        <v>2.541622006929802</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>DO_1_2</t>
+          <t>DO_1_3</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>46015.29166666666</v>
+        <v>46068.79166666666</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>46015.625</v>
+        <v>46069.41666666666</v>
       </c>
       <c r="D10" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E10" t="n">
-        <v>2.754453581023049</v>
+        <v>2.5</v>
       </c>
       <c r="F10" t="n">
-        <v>2.889382418872442</v>
+        <v>2.5</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_step</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>1.006867340116572</v>
+        <v>2.24010207548955</v>
       </c>
     </row>
     <row r="11">
@@ -3449,10 +3959,10 @@
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>45954.20833333334</v>
+        <v>46109.95833333334</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>45954.45833333334</v>
+        <v>46110.20833333334</v>
       </c>
       <c r="D27" t="n">
         <v>7</v>
@@ -3461,15 +3971,15 @@
         <v>2.5</v>
       </c>
       <c r="F27" t="n">
-        <v>2.5</v>
+        <v>2.558879692815726</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Q_step</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H27" t="n">
-        <v>2.24010207548955</v>
+        <v>1.586270319473582</v>
       </c>
     </row>
     <row r="28">
@@ -3479,10 +3989,10 @@
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>46109.95833333334</v>
+        <v>45986.79166666666</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>46110.20833333334</v>
+        <v>45987.04166666666</v>
       </c>
       <c r="D28" t="n">
         <v>7</v>
@@ -3491,15 +4001,15 @@
         <v>2.5</v>
       </c>
       <c r="F28" t="n">
-        <v>2.558879692815726</v>
+        <v>2.5</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_step</t>
         </is>
       </c>
       <c r="H28" t="n">
-        <v>1.586270319473582</v>
+        <v>2.541622006929802</v>
       </c>
     </row>
     <row r="29">
@@ -3509,13 +4019,13 @@
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>45914.25</v>
+        <v>46002.875</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>45926.70833333334</v>
+        <v>46003.08333333334</v>
       </c>
       <c r="D29" t="n">
-        <v>300</v>
+        <v>6</v>
       </c>
       <c r="E29" t="n">
         <v>2.5</v>
@@ -3525,11 +4035,11 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Q_regime</t>
+          <t>Q_step</t>
         </is>
       </c>
       <c r="H29" t="n">
-        <v>1.255262606247016</v>
+        <v>2.866863846995475</v>
       </c>
     </row>
     <row r="30">
@@ -3539,27 +4049,27 @@
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>46069.45833333334</v>
+        <v>45914.25</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>46069.66666666666</v>
+        <v>45923.20833333334</v>
       </c>
       <c r="D30" t="n">
-        <v>6</v>
+        <v>216</v>
       </c>
       <c r="E30" t="n">
-        <v>2.507016709960635</v>
+        <v>2.5</v>
       </c>
       <c r="F30" t="n">
-        <v>2.619198850158543</v>
+        <v>2.5</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_regime</t>
         </is>
       </c>
       <c r="H30" t="n">
-        <v>1.000004982251552</v>
+        <v>1.255262606247016</v>
       </c>
     </row>
     <row r="31">
@@ -3569,27 +4079,27 @@
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>46104.45833333334</v>
+        <v>45953.79166666666</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>46104.875</v>
+        <v>45954.66666666666</v>
       </c>
       <c r="D31" t="n">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="E31" t="n">
-        <v>2.512394845773965</v>
+        <v>2.5</v>
       </c>
       <c r="F31" t="n">
-        <v>2.779489266082209</v>
+        <v>2.5</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_step</t>
         </is>
       </c>
       <c r="H31" t="n">
-        <v>1.09718383978607</v>
+        <v>1.749799171982965</v>
       </c>
     </row>
     <row r="32">
@@ -3599,19 +4109,19 @@
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>46070.20833333334</v>
+        <v>46069.45833333334</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>46070.625</v>
+        <v>46069.66666666666</v>
       </c>
       <c r="D32" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E32" t="n">
-        <v>2.58809163181568</v>
+        <v>2.507016709960635</v>
       </c>
       <c r="F32" t="n">
-        <v>2.643736605693489</v>
+        <v>2.619198850158543</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -3619,7 +4129,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>1.001910606479826</v>
+        <v>1.000004982251552</v>
       </c>
     </row>
     <row r="33">
@@ -3629,19 +4139,19 @@
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>46072.70833333334</v>
+        <v>46104.45833333334</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>46072.91666666666</v>
+        <v>46104.875</v>
       </c>
       <c r="D33" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E33" t="n">
-        <v>2.605294710093437</v>
+        <v>2.512394845773965</v>
       </c>
       <c r="F33" t="n">
-        <v>2.684925504851897</v>
+        <v>2.779489266082209</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -3649,7 +4159,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>1.001865330224722</v>
+        <v>1.09718383978607</v>
       </c>
     </row>
     <row r="34">
@@ -3659,19 +4169,19 @@
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>46015.16666666666</v>
+        <v>46070.20833333334</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>46015.45833333334</v>
+        <v>46070.625</v>
       </c>
       <c r="D34" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E34" t="n">
-        <v>2.632442099658302</v>
+        <v>2.58809163181568</v>
       </c>
       <c r="F34" t="n">
-        <v>2.707099187084153</v>
+        <v>2.643736605693489</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -3679,7 +4189,7 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>1.005069353080617</v>
+        <v>1.001910606479826</v>
       </c>
     </row>
     <row r="35">
@@ -3779,19 +4289,19 @@
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>46029.66666666666</v>
+        <v>46011.5</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>46029.875</v>
+        <v>46011.83333333334</v>
       </c>
       <c r="D38" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E38" t="n">
-        <v>2.365933985321182</v>
+        <v>2.442125375774663</v>
       </c>
       <c r="F38" t="n">
-        <v>2.558276279862052</v>
+        <v>2.50729738658907</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -3799,7 +4309,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>1.001473515745823</v>
+        <v>1.00000001027265</v>
       </c>
     </row>
     <row r="39">
@@ -3809,27 +4319,27 @@
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>46011.5</v>
+        <v>45984.91666666666</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>46011.83333333334</v>
+        <v>45986.33333333334</v>
       </c>
       <c r="D39" t="n">
-        <v>9</v>
+        <v>35</v>
       </c>
       <c r="E39" t="n">
-        <v>2.442125375774663</v>
+        <v>2.5</v>
       </c>
       <c r="F39" t="n">
-        <v>2.50729738658907</v>
+        <v>2.613220978926444</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_step</t>
         </is>
       </c>
       <c r="H39" t="n">
-        <v>1.00000001027265</v>
+        <v>1.229296703595475</v>
       </c>
     </row>
     <row r="40">
@@ -3839,19 +4349,19 @@
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>45984.91666666666</v>
+        <v>46000.625</v>
       </c>
       <c r="C40" s="2" t="n">
-        <v>45985.58333333334</v>
+        <v>46001.04166666666</v>
       </c>
       <c r="D40" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="E40" t="n">
         <v>2.5</v>
       </c>
       <c r="F40" t="n">
-        <v>2.733102015436797</v>
+        <v>2.5</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -3859,7 +4369,7 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>1.229296703595475</v>
+        <v>2.541622006929802</v>
       </c>
     </row>
     <row r="41">
@@ -3989,19 +4499,19 @@
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>46017.375</v>
+        <v>46030.20833333334</v>
       </c>
       <c r="C45" s="2" t="n">
-        <v>46017.83333333334</v>
+        <v>46031.95833333334</v>
       </c>
       <c r="D45" t="n">
-        <v>12</v>
+        <v>43</v>
       </c>
       <c r="E45" t="n">
-        <v>2.167772005843953</v>
+        <v>2.149987352699235</v>
       </c>
       <c r="F45" t="n">
-        <v>2.597986119624171</v>
+        <v>2.3922480432891</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -4009,7 +4519,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>1.000380090649229</v>
+        <v>1.000207179248728</v>
       </c>
     </row>
     <row r="46">
@@ -4019,19 +4529,19 @@
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>46069.75</v>
+        <v>46017.375</v>
       </c>
       <c r="C46" s="2" t="n">
-        <v>46125.70833333334</v>
+        <v>46017.83333333334</v>
       </c>
       <c r="D46" t="n">
-        <v>1344</v>
+        <v>12</v>
       </c>
       <c r="E46" t="n">
-        <v>2.214576517713109</v>
+        <v>2.167772005843953</v>
       </c>
       <c r="F46" t="n">
-        <v>2.496270564148117</v>
+        <v>2.597986119624171</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -4039,7 +4549,7 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>1.00058020526325</v>
+        <v>1.000380090649229</v>
       </c>
     </row>
     <row r="47">
@@ -4049,19 +4559,19 @@
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>46066</v>
+        <v>46069.75</v>
       </c>
       <c r="C47" s="2" t="n">
-        <v>46066.25</v>
+        <v>46077.91666666666</v>
       </c>
       <c r="D47" t="n">
-        <v>7</v>
+        <v>197</v>
       </c>
       <c r="E47" t="n">
-        <v>2.317494233342275</v>
+        <v>2.214576517713109</v>
       </c>
       <c r="F47" t="n">
-        <v>2.505182217827872</v>
+        <v>2.475508943690873</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -4069,7 +4579,7 @@
         </is>
       </c>
       <c r="H47" t="n">
-        <v>1.038916563232165</v>
+        <v>1.00058020526325</v>
       </c>
     </row>
     <row r="48">
@@ -4079,27 +4589,27 @@
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>46018</v>
+        <v>46032.41666666666</v>
       </c>
       <c r="C48" s="2" t="n">
-        <v>46038.25</v>
+        <v>46032.625</v>
       </c>
       <c r="D48" t="n">
-        <v>487</v>
+        <v>6</v>
       </c>
       <c r="E48" t="n">
-        <v>2.317959986394953</v>
+        <v>2.256477025195484</v>
       </c>
       <c r="F48" t="n">
-        <v>2.497788572677653</v>
+        <v>2.321600742859642</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Q_regime</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H48" t="n">
-        <v>1.081134041730266</v>
+        <v>1.088169856401719</v>
       </c>
     </row>
     <row r="49">
@@ -4109,19 +4619,19 @@
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>46063.875</v>
+        <v>46066</v>
       </c>
       <c r="C49" s="2" t="n">
-        <v>46064.08333333334</v>
+        <v>46066.25</v>
       </c>
       <c r="D49" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>2.46371245656945</v>
+        <v>2.317494233342275</v>
       </c>
       <c r="F49" t="n">
-        <v>2.641043884053045</v>
+        <v>2.505182217827872</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -4129,7 +4639,7 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>1.010767658751164</v>
+        <v>1.038916563232165</v>
       </c>
     </row>
     <row r="50">
@@ -4139,27 +4649,27 @@
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>46067.33333333334</v>
+        <v>46018</v>
       </c>
       <c r="C50" s="2" t="n">
-        <v>46067.54166666666</v>
+        <v>46025.20833333334</v>
       </c>
       <c r="D50" t="n">
-        <v>6</v>
+        <v>174</v>
       </c>
       <c r="E50" t="n">
-        <v>2.651713442492882</v>
+        <v>2.317959986394953</v>
       </c>
       <c r="F50" t="n">
-        <v>2.772109368538855</v>
+        <v>2.492738182474997</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_regime</t>
         </is>
       </c>
       <c r="H50" t="n">
-        <v>1.056283906171612</v>
+        <v>1.081134041730266</v>
       </c>
     </row>
     <row r="51">
@@ -4169,19 +4679,19 @@
         </is>
       </c>
       <c r="B51" s="2" t="n">
-        <v>46011.91666666666</v>
+        <v>46118.41666666666</v>
       </c>
       <c r="C51" s="2" t="n">
-        <v>46012.125</v>
+        <v>46122.45833333334</v>
       </c>
       <c r="D51" t="n">
-        <v>6</v>
+        <v>98</v>
       </c>
       <c r="E51" t="n">
-        <v>2.737078226139449</v>
+        <v>2.338714230036328</v>
       </c>
       <c r="F51" t="n">
-        <v>2.847472325151764</v>
+        <v>2.505987799864467</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -4189,97 +4699,97 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>1.000313907608093</v>
+        <v>1.04046058341234</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>ORP_1_3</t>
+          <t>ORP_1_2</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
-        <v>45946.75</v>
+        <v>46033.625</v>
       </c>
       <c r="C52" s="2" t="n">
-        <v>45951.5</v>
+        <v>46038.25</v>
       </c>
       <c r="D52" t="n">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="E52" t="n">
-        <v>2.5</v>
+        <v>2.352648455999176</v>
       </c>
       <c r="F52" t="n">
-        <v>2.5</v>
+        <v>2.505656680806336</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Q_step</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H52" t="n">
-        <v>2.058379058668964</v>
+        <v>1.10286685173526</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ORP_1_3</t>
+          <t>ORP_1_2</t>
         </is>
       </c>
       <c r="B53" s="2" t="n">
-        <v>45945.25</v>
+        <v>46115</v>
       </c>
       <c r="C53" s="2" t="n">
-        <v>45945.45833333334</v>
+        <v>46115.29166666666</v>
       </c>
       <c r="D53" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E53" t="n">
-        <v>2.5</v>
+        <v>2.356657639501725</v>
       </c>
       <c r="F53" t="n">
-        <v>2.5</v>
+        <v>2.524522307136362</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Q_regime</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H53" t="n">
-        <v>1.961678843667339</v>
+        <v>1.102732526289897</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ORP_1_3</t>
+          <t>ORP_1_2</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
-        <v>45985.79166666666</v>
+        <v>46082.25</v>
       </c>
       <c r="C54" s="2" t="n">
-        <v>45986.125</v>
+        <v>46088.45833333334</v>
       </c>
       <c r="D54" t="n">
-        <v>9</v>
+        <v>150</v>
       </c>
       <c r="E54" t="n">
-        <v>2.564243254468536</v>
+        <v>2.370479410035172</v>
       </c>
       <c r="F54" t="n">
-        <v>2.759940853427584</v>
+        <v>2.498346242527374</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Q_step</t>
+          <t>Q_regime</t>
         </is>
       </c>
       <c r="H54" t="n">
-        <v>1.229296703595475</v>
+        <v>1.333577532071762</v>
       </c>
     </row>
     <row r="55">
@@ -4289,19 +4799,19 @@
         </is>
       </c>
       <c r="B55" s="2" t="n">
-        <v>45945.79166666666</v>
+        <v>45944.25</v>
       </c>
       <c r="C55" s="2" t="n">
-        <v>45946.20833333334</v>
+        <v>45944.79166666666</v>
       </c>
       <c r="D55" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E55" t="n">
-        <v>2.635659596744977</v>
+        <v>2.378602582433596</v>
       </c>
       <c r="F55" t="n">
-        <v>2.812160783667882</v>
+        <v>2.65933923989452</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -4309,7 +4819,7 @@
         </is>
       </c>
       <c r="H55" t="n">
-        <v>2.058379058668964</v>
+        <v>1.282329482970322</v>
       </c>
     </row>
     <row r="56">
@@ -4319,19 +4829,19 @@
         </is>
       </c>
       <c r="B56" s="2" t="n">
-        <v>45944.45833333334</v>
+        <v>45986.66666666666</v>
       </c>
       <c r="C56" s="2" t="n">
-        <v>45944.70833333334</v>
+        <v>45987.08333333334</v>
       </c>
       <c r="D56" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E56" t="n">
-        <v>2.681541950564857</v>
+        <v>2.5</v>
       </c>
       <c r="F56" t="n">
-        <v>2.782221389952219</v>
+        <v>2.5</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
@@ -4339,7 +4849,7 @@
         </is>
       </c>
       <c r="H56" t="n">
-        <v>1.282329482970322</v>
+        <v>2.541622006929802</v>
       </c>
     </row>
     <row r="57">
@@ -4349,19 +4859,19 @@
         </is>
       </c>
       <c r="B57" s="2" t="n">
-        <v>46014.45833333334</v>
+        <v>45948.875</v>
       </c>
       <c r="C57" s="2" t="n">
-        <v>46014.75</v>
+        <v>45949.83333333334</v>
       </c>
       <c r="D57" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="E57" t="n">
-        <v>2.838559067395091</v>
+        <v>2.5</v>
       </c>
       <c r="F57" t="n">
-        <v>2.919989230357585</v>
+        <v>2.5</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -4369,7 +4879,7 @@
         </is>
       </c>
       <c r="H57" t="n">
-        <v>1.51542430420249</v>
+        <v>2.648143459082469</v>
       </c>
     </row>
     <row r="58">
@@ -4379,177 +4889,387 @@
         </is>
       </c>
       <c r="B58" s="2" t="n">
-        <v>45912.20833333334</v>
+        <v>45946.33333333334</v>
       </c>
       <c r="C58" s="2" t="n">
-        <v>45912.41666666666</v>
+        <v>45948.375</v>
       </c>
       <c r="D58" t="n">
-        <v>6</v>
+        <v>50</v>
       </c>
       <c r="E58" t="n">
-        <v>2.838808585782044</v>
+        <v>2.5</v>
       </c>
       <c r="F58" t="n">
-        <v>2.916402563418345</v>
+        <v>2.5</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Q_step</t>
+          <t>Q_regime</t>
         </is>
       </c>
       <c r="H58" t="n">
-        <v>1.51542430420249</v>
+        <v>2.108098132368428</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>ORP_2_1</t>
+          <t>ORP_1_3</t>
         </is>
       </c>
       <c r="B59" s="2" t="n">
-        <v>46083.5</v>
+        <v>45945.08333333334</v>
       </c>
       <c r="C59" s="2" t="n">
-        <v>46083.75</v>
+        <v>45945.45833333334</v>
       </c>
       <c r="D59" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>2.469548897143255</v>
+        <v>2.5</v>
       </c>
       <c r="F59" t="n">
-        <v>2.675205925395538</v>
+        <v>2.644339225428953</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_regime</t>
         </is>
       </c>
       <c r="H59" t="n">
-        <v>1.09003124068793</v>
+        <v>1.961678843667339</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ORP_2_1</t>
+          <t>ORP_1_3</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
-        <v>46014.41666666666</v>
+        <v>45940.54166666666</v>
       </c>
       <c r="C60" s="2" t="n">
-        <v>46014.66666666666</v>
+        <v>45941.25</v>
       </c>
       <c r="D60" t="n">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="E60" t="n">
-        <v>2.741435296101974</v>
+        <v>2.5</v>
       </c>
       <c r="F60" t="n">
-        <v>2.849723924600531</v>
+        <v>2.5</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_step</t>
         </is>
       </c>
       <c r="H60" t="n">
-        <v>1.180759797519993</v>
+        <v>2.437776348413636</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>ORP_2_1</t>
+          <t>ORP_1_3</t>
         </is>
       </c>
       <c r="B61" s="2" t="n">
-        <v>45912.625</v>
+        <v>45985.79166666666</v>
       </c>
       <c r="C61" s="2" t="n">
-        <v>45912.83333333334</v>
+        <v>45986.125</v>
       </c>
       <c r="D61" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E61" t="n">
-        <v>2.758076189060307</v>
+        <v>2.564243254468536</v>
       </c>
       <c r="F61" t="n">
-        <v>2.80686385338087</v>
+        <v>2.759940853427584</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_step</t>
         </is>
       </c>
       <c r="H61" t="n">
-        <v>1.00539930261449</v>
+        <v>1.229296703595475</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ORP_2_2</t>
+          <t>ORP_1_3</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
-        <v>46119</v>
+        <v>45945.79166666666</v>
       </c>
       <c r="C62" s="2" t="n">
-        <v>46125.70833333334</v>
+        <v>45946.20833333334</v>
       </c>
       <c r="D62" t="n">
-        <v>162</v>
+        <v>11</v>
       </c>
       <c r="E62" t="n">
-        <v>2.416818111700139</v>
+        <v>2.635659596744977</v>
       </c>
       <c r="F62" t="n">
-        <v>2.499486531553705</v>
+        <v>2.812160783667882</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Q_regime</t>
+          <t>Q_step</t>
         </is>
       </c>
       <c r="H62" t="n">
-        <v>1.160462951377068</v>
+        <v>2.058379058668964</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
+          <t>ORP_1_3</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="n">
+        <v>45912.16666666666</v>
+      </c>
+      <c r="C63" s="2" t="n">
+        <v>45912.41666666666</v>
+      </c>
+      <c r="D63" t="n">
+        <v>7</v>
+      </c>
+      <c r="E63" t="n">
+        <v>2.81451481117033</v>
+      </c>
+      <c r="F63" t="n">
+        <v>2.878204171198647</v>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Q_step</t>
+        </is>
+      </c>
+      <c r="H63" t="n">
+        <v>1.51542430420249</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>ORP_1_3</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="n">
+        <v>46014.45833333334</v>
+      </c>
+      <c r="C64" s="2" t="n">
+        <v>46014.75</v>
+      </c>
+      <c r="D64" t="n">
+        <v>8</v>
+      </c>
+      <c r="E64" t="n">
+        <v>2.838559067395091</v>
+      </c>
+      <c r="F64" t="n">
+        <v>2.919989230357585</v>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Q_step</t>
+        </is>
+      </c>
+      <c r="H64" t="n">
+        <v>1.51542430420249</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>ORP_2_1</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="n">
+        <v>46083.5</v>
+      </c>
+      <c r="C65" s="2" t="n">
+        <v>46083.75</v>
+      </c>
+      <c r="D65" t="n">
+        <v>7</v>
+      </c>
+      <c r="E65" t="n">
+        <v>2.469548897143255</v>
+      </c>
+      <c r="F65" t="n">
+        <v>2.675205925395538</v>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Q_drift</t>
+        </is>
+      </c>
+      <c r="H65" t="n">
+        <v>1.09003124068793</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>ORP_2_1</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="n">
+        <v>46014.41666666666</v>
+      </c>
+      <c r="C66" s="2" t="n">
+        <v>46014.66666666666</v>
+      </c>
+      <c r="D66" t="n">
+        <v>7</v>
+      </c>
+      <c r="E66" t="n">
+        <v>2.741435296101974</v>
+      </c>
+      <c r="F66" t="n">
+        <v>2.849723924600531</v>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Q_drift</t>
+        </is>
+      </c>
+      <c r="H66" t="n">
+        <v>1.180759797519993</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>ORP_2_1</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="n">
+        <v>45912.625</v>
+      </c>
+      <c r="C67" s="2" t="n">
+        <v>45912.83333333334</v>
+      </c>
+      <c r="D67" t="n">
+        <v>6</v>
+      </c>
+      <c r="E67" t="n">
+        <v>2.758076189060307</v>
+      </c>
+      <c r="F67" t="n">
+        <v>2.80686385338087</v>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Q_drift</t>
+        </is>
+      </c>
+      <c r="H67" t="n">
+        <v>1.00539930261449</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
           <t>ORP_2_2</t>
         </is>
       </c>
-      <c r="B63" s="2" t="n">
+      <c r="B68" s="2" t="n">
+        <v>46119</v>
+      </c>
+      <c r="C68" s="2" t="n">
+        <v>46122.45833333334</v>
+      </c>
+      <c r="D68" t="n">
+        <v>84</v>
+      </c>
+      <c r="E68" t="n">
+        <v>2.416818111700139</v>
+      </c>
+      <c r="F68" t="n">
+        <v>2.499009739425002</v>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Q_regime</t>
+        </is>
+      </c>
+      <c r="H68" t="n">
+        <v>1.160462951377068</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>ORP_2_2</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="n">
         <v>46036.75</v>
       </c>
-      <c r="C63" s="2" t="n">
+      <c r="C69" s="2" t="n">
         <v>46037.45833333334</v>
       </c>
-      <c r="D63" t="n">
+      <c r="D69" t="n">
         <v>18</v>
       </c>
-      <c r="E63" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="F63" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="G63" t="inlineStr">
+      <c r="E69" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F69" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G69" t="inlineStr">
         <is>
           <t>Q_regime</t>
         </is>
       </c>
-      <c r="H63" t="n">
+      <c r="H69" t="n">
         <v>1.922445730625928</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>ORP_2_2</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="n">
+        <v>46070.33333333334</v>
+      </c>
+      <c r="C70" s="2" t="n">
+        <v>46070.75</v>
+      </c>
+      <c r="D70" t="n">
+        <v>11</v>
+      </c>
+      <c r="E70" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F70" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Q_step</t>
+        </is>
+      </c>
+      <c r="H70" t="n">
+        <v>2.866863846995475</v>
       </c>
     </row>
   </sheetData>
@@ -4563,7 +5283,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4626,13 +5346,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D3" t="n">
-        <v>47</v>
+        <v>220</v>
       </c>
       <c r="E3" t="n">
-        <v>2.633566080602755</v>
+        <v>2.504552591965269</v>
       </c>
     </row>
     <row r="4">
@@ -4643,38 +5363,38 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Q_regime</t>
+          <t>Q_step</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D4" t="n">
-        <v>209</v>
+        <v>28</v>
       </c>
       <c r="E4" t="n">
-        <v>2.471022684808087</v>
+        <v>2.575342961439494</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DO_1_2</t>
+          <t>DO_1_3</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Q_step</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="C5" t="n">
         <v>2</v>
       </c>
       <c r="D5" t="n">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="E5" t="n">
-        <v>2.659995022040581</v>
+        <v>2.744974235338862</v>
       </c>
     </row>
     <row r="6">
@@ -4685,17 +5405,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_step</t>
         </is>
       </c>
       <c r="C6" t="n">
         <v>2</v>
       </c>
       <c r="D6" t="n">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="E6" t="n">
-        <v>2.744974235338862</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="7">
@@ -4773,13 +5493,13 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D10" t="n">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="E10" t="n">
-        <v>2.572306757539529</v>
+        <v>2.62222065404098</v>
       </c>
     </row>
     <row r="11">
@@ -4797,7 +5517,7 @@
         <v>1</v>
       </c>
       <c r="D11" t="n">
-        <v>300</v>
+        <v>216</v>
       </c>
       <c r="E11" t="n">
         <v>2.5</v>
@@ -4815,10 +5535,10 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D12" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="E12" t="n">
         <v>2.5</v>
@@ -4836,13 +5556,13 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D13" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="E13" t="n">
-        <v>2.479349502160271</v>
+        <v>2.490691053844179</v>
       </c>
     </row>
     <row r="14">
@@ -4857,13 +5577,13 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D14" t="n">
-        <v>24</v>
+        <v>63</v>
       </c>
       <c r="E14" t="n">
-        <v>2.521818719159612</v>
+        <v>2.567758341951052</v>
       </c>
     </row>
     <row r="15">
@@ -4878,13 +5598,13 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="D15" t="n">
-        <v>1381</v>
+        <v>602</v>
       </c>
       <c r="E15" t="n">
-        <v>2.425391147016853</v>
+        <v>2.382885255766381</v>
       </c>
     </row>
     <row r="16">
@@ -4899,13 +5619,13 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D16" t="n">
-        <v>487</v>
+        <v>373</v>
       </c>
       <c r="E16" t="n">
-        <v>2.317959986394953</v>
+        <v>2.396146465476709</v>
       </c>
     </row>
     <row r="17">
@@ -4920,10 +5640,10 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D17" t="n">
-        <v>6</v>
+        <v>60</v>
       </c>
       <c r="E17" t="n">
         <v>2.5</v>
@@ -4941,13 +5661,13 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D18" t="n">
-        <v>156</v>
+        <v>102</v>
       </c>
       <c r="E18" t="n">
-        <v>2.676468742492584</v>
+        <v>2.591447414026566</v>
       </c>
     </row>
     <row r="19">
@@ -4986,10 +5706,31 @@
         <v>2</v>
       </c>
       <c r="D20" t="n">
-        <v>180</v>
+        <v>102</v>
       </c>
       <c r="E20" t="n">
         <v>2.45840905585007</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>ORP_2_2</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Q_step</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" t="n">
+        <v>11</v>
+      </c>
+      <c r="E21" t="n">
+        <v>2.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix D1 topology-constrained PLS peers
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D1 Sensor health/outputs/data/D1_event_windows.xlsx
+++ b/Project 1 Data Quality Assessment/D1 Sensor health/outputs/data/D1_event_windows.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H82"/>
+  <dimension ref="A1:H89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -492,10 +492,10 @@
         <v>7</v>
       </c>
       <c r="E2" t="n">
-        <v>2.776674147507447</v>
+        <v>2.778023496646145</v>
       </c>
       <c r="F2" t="n">
-        <v>2.84874268532911</v>
+        <v>2.849906663019707</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>1.000005614214015</v>
+        <v>1.000005525074796</v>
       </c>
     </row>
     <row r="3">
@@ -522,10 +522,10 @@
         <v>6</v>
       </c>
       <c r="E3" t="n">
-        <v>2.82166051957243</v>
+        <v>2.817097209666348</v>
       </c>
       <c r="F3" t="n">
-        <v>2.955211575393891</v>
+        <v>2.950866201389108</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>1.084277888278427</v>
+        <v>1.078295198584504</v>
       </c>
     </row>
     <row r="4">
@@ -1302,10 +1302,10 @@
         <v>6</v>
       </c>
       <c r="E29" t="n">
-        <v>2.830483355621616</v>
+        <v>2.825158860728377</v>
       </c>
       <c r="F29" t="n">
-        <v>2.89598059026946</v>
+        <v>2.879490557669677</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -1313,7 +1313,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>1.017865000497111</v>
+        <v>1.006655537563976</v>
       </c>
     </row>
     <row r="30">
@@ -1332,10 +1332,10 @@
         <v>6</v>
       </c>
       <c r="E30" t="n">
-        <v>2.809240006043018</v>
+        <v>2.809293725156838</v>
       </c>
       <c r="F30" t="n">
-        <v>2.855236973622998</v>
+        <v>2.853676095959244</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1343,7 +1343,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>1.000329158340358</v>
+        <v>1.000680342465465</v>
       </c>
     </row>
     <row r="31">
@@ -1362,10 +1362,10 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>2.807613851151439</v>
+        <v>2.810519000303214</v>
       </c>
       <c r="F31" t="n">
-        <v>2.862055297206406</v>
+        <v>2.853831015240609</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>1.00472076843603</v>
+        <v>1.005044614206155</v>
       </c>
     </row>
     <row r="32">
@@ -1392,10 +1392,10 @@
         <v>8</v>
       </c>
       <c r="E32" t="n">
-        <v>2.631283258737578</v>
+        <v>2.631677867231224</v>
       </c>
       <c r="F32" t="n">
-        <v>2.86650035514931</v>
+        <v>2.867962299653354</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -1403,7 +1403,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>1.000395008168533</v>
+        <v>1.002561889542912</v>
       </c>
     </row>
     <row r="33">
@@ -1413,19 +1413,19 @@
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>45982.66666666666</v>
+        <v>45952</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>45983.45833333334</v>
+        <v>45952.29166666666</v>
       </c>
       <c r="D33" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="E33" t="n">
-        <v>2.590874993410552</v>
+        <v>2.721496201402909</v>
       </c>
       <c r="F33" t="n">
-        <v>2.842002306336331</v>
+        <v>2.868353618291169</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -1433,7 +1433,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>1.000001443244321</v>
+        <v>1.002264254450091</v>
       </c>
     </row>
     <row r="34">
@@ -1443,19 +1443,19 @@
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>45984.45833333334</v>
+        <v>45982.625</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>45984.91666666666</v>
+        <v>45983.41666666666</v>
       </c>
       <c r="D34" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="E34" t="n">
-        <v>2.447921818153538</v>
+        <v>2.593590713815669</v>
       </c>
       <c r="F34" t="n">
-        <v>2.717737062928489</v>
+        <v>2.824028653460144</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -1463,7 +1463,7 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>1.00000065855702</v>
+        <v>1.000004535023473</v>
       </c>
     </row>
     <row r="35">
@@ -1473,27 +1473,27 @@
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>45985</v>
+        <v>45984.45833333334</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>45985.54166666666</v>
+        <v>45984.91666666666</v>
       </c>
       <c r="D35" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E35" t="n">
-        <v>2.550175579847397</v>
+        <v>2.447935866890584</v>
       </c>
       <c r="F35" t="n">
-        <v>2.71946138852274</v>
+        <v>2.718102655457825</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Q_step</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H35" t="n">
-        <v>1.156662891187058</v>
+        <v>1.000001103825005</v>
       </c>
     </row>
     <row r="36">
@@ -1503,27 +1503,27 @@
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>46011.45833333334</v>
+        <v>45985</v>
       </c>
       <c r="C36" s="2" t="n">
-        <v>46011.83333333334</v>
+        <v>45985.54166666666</v>
       </c>
       <c r="D36" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E36" t="n">
-        <v>2.567188046035585</v>
+        <v>2.550175579847397</v>
       </c>
       <c r="F36" t="n">
-        <v>2.646585973935476</v>
+        <v>2.71946138852274</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_step</t>
         </is>
       </c>
       <c r="H36" t="n">
-        <v>1.000000028806149</v>
+        <v>1.156662891187058</v>
       </c>
     </row>
     <row r="37">
@@ -1533,19 +1533,19 @@
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>46011.91666666666</v>
+        <v>45998.66666666666</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>46012.125</v>
+        <v>45998.875</v>
       </c>
       <c r="D37" t="n">
         <v>6</v>
       </c>
       <c r="E37" t="n">
-        <v>2.400909013242728</v>
+        <v>2.211936251292717</v>
       </c>
       <c r="F37" t="n">
-        <v>2.583739404377635</v>
+        <v>2.479658830044532</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -1553,7 +1553,7 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>1.000005203420343</v>
+        <v>1.0189217456638</v>
       </c>
     </row>
     <row r="38">
@@ -1563,19 +1563,19 @@
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>46013.66666666666</v>
+        <v>46011.5</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>46014.20833333334</v>
+        <v>46011.83333333334</v>
       </c>
       <c r="D38" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E38" t="n">
-        <v>2.451291985467262</v>
+        <v>2.567194367272065</v>
       </c>
       <c r="F38" t="n">
-        <v>2.67249520178254</v>
+        <v>2.64530938286319</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -1583,7 +1583,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>1.000000000738104</v>
+        <v>1.000000067627254</v>
       </c>
     </row>
     <row r="39">
@@ -1593,27 +1593,27 @@
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>46014.45833333334</v>
+        <v>46011.91666666666</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>46014.66666666666</v>
+        <v>46012.20833333334</v>
       </c>
       <c r="D39" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E39" t="n">
-        <v>2.776726839400139</v>
+        <v>2.392805004675806</v>
       </c>
       <c r="F39" t="n">
-        <v>2.819586287662029</v>
+        <v>2.596736357047955</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Q_step</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H39" t="n">
-        <v>1.535711553296295</v>
+        <v>1.000015078979207</v>
       </c>
     </row>
     <row r="40">
@@ -1623,79 +1623,79 @@
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>46102.91666666666</v>
+        <v>46013.66666666666</v>
       </c>
       <c r="C40" s="2" t="n">
-        <v>46103.33333333334</v>
+        <v>46014.16666666666</v>
       </c>
       <c r="D40" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E40" t="n">
-        <v>2</v>
+        <v>2.451277291557278</v>
       </c>
       <c r="F40" t="n">
-        <v>2.081402219039941</v>
+        <v>2.664274531537799</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Q_freeze</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H40" t="n">
-        <v>1.226970741004972</v>
+        <v>1.000000000141117</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ORP_1_1</t>
+          <t>DO_2_4</t>
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>45920.16666666666</v>
+        <v>46014.45833333334</v>
       </c>
       <c r="C41" s="2" t="n">
-        <v>45920.375</v>
+        <v>46014.66666666666</v>
       </c>
       <c r="D41" t="n">
         <v>6</v>
       </c>
       <c r="E41" t="n">
-        <v>2.757376328495986</v>
+        <v>2.776726839400139</v>
       </c>
       <c r="F41" t="n">
-        <v>2.879726012342237</v>
+        <v>2.819586287662029</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_step</t>
         </is>
       </c>
       <c r="H41" t="n">
-        <v>1.000007312976706</v>
+        <v>1.535711553296295</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ORP_1_1</t>
+          <t>DO_2_4</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>45972.875</v>
+        <v>46029.625</v>
       </c>
       <c r="C42" s="2" t="n">
-        <v>45973.125</v>
+        <v>46029.875</v>
       </c>
       <c r="D42" t="n">
         <v>7</v>
       </c>
       <c r="E42" t="n">
-        <v>2.809682021993101</v>
+        <v>2.567062194481823</v>
       </c>
       <c r="F42" t="n">
-        <v>2.874583149247187</v>
+        <v>2.755760587104711</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -1703,59 +1703,59 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>1.000251210791262</v>
+        <v>1.001531969385012</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ORP_1_1</t>
+          <t>DO_2_4</t>
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>46031.41666666666</v>
+        <v>46064.29166666666</v>
       </c>
       <c r="C43" s="2" t="n">
-        <v>46031.625</v>
+        <v>46064.5</v>
       </c>
       <c r="D43" t="n">
         <v>6</v>
       </c>
       <c r="E43" t="n">
-        <v>2.834374417406643</v>
+        <v>2.682590823715822</v>
       </c>
       <c r="F43" t="n">
-        <v>2.888146187617946</v>
+        <v>2.766922847811539</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_spike</t>
         </is>
       </c>
       <c r="H43" t="n">
-        <v>1.012556226373021</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ORP_1_1</t>
+          <t>DO_2_4</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>46069.70833333334</v>
+        <v>46068.75</v>
       </c>
       <c r="C44" s="2" t="n">
-        <v>46070.08333333334</v>
+        <v>46069.125</v>
       </c>
       <c r="D44" t="n">
         <v>10</v>
       </c>
       <c r="E44" t="n">
-        <v>2.896610077643929</v>
+        <v>2.534498966663721</v>
       </c>
       <c r="F44" t="n">
-        <v>2.925288845222536</v>
+        <v>2.670607565166778</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -1763,29 +1763,29 @@
         </is>
       </c>
       <c r="H44" t="n">
-        <v>1.000175276400918</v>
+        <v>1.029970506055951</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ORP_1_1</t>
+          <t>DO_2_4</t>
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>46070.66666666666</v>
+        <v>46070.29166666666</v>
       </c>
       <c r="C45" s="2" t="n">
-        <v>46070.875</v>
+        <v>46070.5</v>
       </c>
       <c r="D45" t="n">
         <v>6</v>
       </c>
       <c r="E45" t="n">
-        <v>2.862447879436455</v>
+        <v>2.703520320400192</v>
       </c>
       <c r="F45" t="n">
-        <v>2.904058513690617</v>
+        <v>2.844309062842978</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -1793,29 +1793,29 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>1.000000824987803</v>
+        <v>1.230426783607971</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ORP_1_1</t>
+          <t>DO_2_4</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>46071.16666666666</v>
+        <v>46077.70833333334</v>
       </c>
       <c r="C46" s="2" t="n">
-        <v>46071.375</v>
+        <v>46078</v>
       </c>
       <c r="D46" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E46" t="n">
-        <v>2.848990227837606</v>
+        <v>2.588607853112589</v>
       </c>
       <c r="F46" t="n">
-        <v>2.89291995286294</v>
+        <v>2.84003479810486</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -1823,29 +1823,29 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>1.000000054774468</v>
+        <v>1.03956381193685</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>ORP_1_1</t>
+          <t>DO_2_4</t>
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>46072.875</v>
+        <v>46102.875</v>
       </c>
       <c r="C47" s="2" t="n">
-        <v>46073.08333333334</v>
+        <v>46103.33333333334</v>
       </c>
       <c r="D47" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E47" t="n">
-        <v>2.657825556091456</v>
+        <v>2</v>
       </c>
       <c r="F47" t="n">
-        <v>2.816614046922334</v>
+        <v>2.114764389726374</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -1853,29 +1853,29 @@
         </is>
       </c>
       <c r="H47" t="n">
-        <v>1.000210598230002</v>
+        <v>1.000081729568714</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>ORP_1_1</t>
+          <t>DO_2_4</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>46078.33333333334</v>
+        <v>46103.70833333334</v>
       </c>
       <c r="C48" s="2" t="n">
-        <v>46078.625</v>
+        <v>46104.08333333334</v>
       </c>
       <c r="D48" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E48" t="n">
-        <v>2.746832855958405</v>
+        <v>2.677584717833867</v>
       </c>
       <c r="F48" t="n">
-        <v>2.824440399192632</v>
+        <v>2.780025940040364</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -1883,7 +1883,7 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>1.001550894467055</v>
+        <v>1.000844426489696</v>
       </c>
     </row>
     <row r="49">
@@ -1893,19 +1893,19 @@
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>46094.375</v>
+        <v>45920.16666666666</v>
       </c>
       <c r="C49" s="2" t="n">
-        <v>46094.58333333334</v>
+        <v>45920.375</v>
       </c>
       <c r="D49" t="n">
         <v>6</v>
       </c>
       <c r="E49" t="n">
-        <v>2.838629155558616</v>
+        <v>2.757376328495986</v>
       </c>
       <c r="F49" t="n">
-        <v>2.891784470303272</v>
+        <v>2.879726012342237</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -1913,7 +1913,7 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>1.019566742923476</v>
+        <v>1.000007312976706</v>
       </c>
     </row>
     <row r="50">
@@ -1923,19 +1923,19 @@
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>46103.5</v>
+        <v>45972.875</v>
       </c>
       <c r="C50" s="2" t="n">
-        <v>46103.75</v>
+        <v>45973.125</v>
       </c>
       <c r="D50" t="n">
         <v>7</v>
       </c>
       <c r="E50" t="n">
-        <v>2.894842078739759</v>
+        <v>2.809682021993101</v>
       </c>
       <c r="F50" t="n">
-        <v>2.932507636981506</v>
+        <v>2.874583149247187</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -1943,7 +1943,7 @@
         </is>
       </c>
       <c r="H50" t="n">
-        <v>1.001234465516338</v>
+        <v>1.000251210791262</v>
       </c>
     </row>
     <row r="51">
@@ -1953,19 +1953,19 @@
         </is>
       </c>
       <c r="B51" s="2" t="n">
-        <v>46114.95833333334</v>
+        <v>46031.41666666666</v>
       </c>
       <c r="C51" s="2" t="n">
-        <v>46115.33333333334</v>
+        <v>46031.625</v>
       </c>
       <c r="D51" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E51" t="n">
-        <v>2.798742539278037</v>
+        <v>2.834374417406643</v>
       </c>
       <c r="F51" t="n">
-        <v>2.860378239024466</v>
+        <v>2.888146187617946</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>1.000170122637875</v>
+        <v>1.012556226373021</v>
       </c>
     </row>
     <row r="52">
@@ -1983,19 +1983,19 @@
         </is>
       </c>
       <c r="B52" s="2" t="n">
-        <v>46115.70833333334</v>
+        <v>46069.70833333334</v>
       </c>
       <c r="C52" s="2" t="n">
-        <v>46115.91666666666</v>
+        <v>46070.08333333334</v>
       </c>
       <c r="D52" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>2.82685896567884</v>
+        <v>2.896610077643929</v>
       </c>
       <c r="F52" t="n">
-        <v>2.865204925287654</v>
+        <v>2.925288845222536</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -2003,7 +2003,7 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>1.005129204816508</v>
+        <v>1.000175276400918</v>
       </c>
     </row>
     <row r="53">
@@ -2013,19 +2013,19 @@
         </is>
       </c>
       <c r="B53" s="2" t="n">
-        <v>46117.58333333334</v>
+        <v>46070.66666666666</v>
       </c>
       <c r="C53" s="2" t="n">
-        <v>46117.79166666666</v>
+        <v>46070.875</v>
       </c>
       <c r="D53" t="n">
         <v>6</v>
       </c>
       <c r="E53" t="n">
-        <v>2.722453332391307</v>
+        <v>2.862447879436455</v>
       </c>
       <c r="F53" t="n">
-        <v>2.800563384417298</v>
+        <v>2.904058513690617</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -2033,29 +2033,29 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>1.014371043248799</v>
+        <v>1.000000824987803</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ORP_1_2</t>
+          <t>ORP_1_1</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
-        <v>46011.91666666666</v>
+        <v>46071.16666666666</v>
       </c>
       <c r="C54" s="2" t="n">
-        <v>46012.29166666666</v>
+        <v>46071.375</v>
       </c>
       <c r="D54" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E54" t="n">
-        <v>2.757755442063062</v>
+        <v>2.848990227837606</v>
       </c>
       <c r="F54" t="n">
-        <v>2.872621839265668</v>
+        <v>2.89291995286294</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -2063,29 +2063,29 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>1.00000034906757</v>
+        <v>1.000000054774468</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>ORP_1_2</t>
+          <t>ORP_1_1</t>
         </is>
       </c>
       <c r="B55" s="2" t="n">
-        <v>46013.41666666666</v>
+        <v>46072.875</v>
       </c>
       <c r="C55" s="2" t="n">
-        <v>46013.75</v>
+        <v>46073.08333333334</v>
       </c>
       <c r="D55" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E55" t="n">
-        <v>2.544626382375943</v>
+        <v>2.657825556091456</v>
       </c>
       <c r="F55" t="n">
-        <v>2.775858446615649</v>
+        <v>2.816614046922334</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -2093,29 +2093,29 @@
         </is>
       </c>
       <c r="H55" t="n">
-        <v>1.000011018866541</v>
+        <v>1.000210598230002</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>ORP_1_2</t>
+          <t>ORP_1_1</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
-        <v>46015.375</v>
+        <v>46078.33333333334</v>
       </c>
       <c r="C56" s="2" t="n">
-        <v>46015.625</v>
+        <v>46078.625</v>
       </c>
       <c r="D56" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E56" t="n">
-        <v>2.692135104591072</v>
+        <v>2.746832855958405</v>
       </c>
       <c r="F56" t="n">
-        <v>2.751468079267666</v>
+        <v>2.824440399192632</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
@@ -2123,29 +2123,29 @@
         </is>
       </c>
       <c r="H56" t="n">
-        <v>1.001428473812057</v>
+        <v>1.001550894467055</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ORP_1_2</t>
+          <t>ORP_1_1</t>
         </is>
       </c>
       <c r="B57" s="2" t="n">
-        <v>46017.33333333334</v>
+        <v>46094.375</v>
       </c>
       <c r="C57" s="2" t="n">
-        <v>46017.79166666666</v>
+        <v>46094.58333333334</v>
       </c>
       <c r="D57" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E57" t="n">
-        <v>2.38724600616407</v>
+        <v>2.838629155558616</v>
       </c>
       <c r="F57" t="n">
-        <v>2.584654464869179</v>
+        <v>2.891784470303272</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -2153,59 +2153,59 @@
         </is>
       </c>
       <c r="H57" t="n">
-        <v>1.000000453251144</v>
+        <v>1.019566742923476</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ORP_1_2</t>
+          <t>ORP_1_1</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
-        <v>46018</v>
+        <v>46103.5</v>
       </c>
       <c r="C58" s="2" t="n">
-        <v>46028.29166666666</v>
+        <v>46103.75</v>
       </c>
       <c r="D58" t="n">
-        <v>248</v>
+        <v>7</v>
       </c>
       <c r="E58" t="n">
-        <v>2.5</v>
+        <v>2.894842078739759</v>
       </c>
       <c r="F58" t="n">
-        <v>2.5</v>
+        <v>2.932507636981506</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Q_regime</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H58" t="n">
-        <v>1.081134041730266</v>
+        <v>1.001234465516338</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>ORP_1_2</t>
+          <t>ORP_1_1</t>
         </is>
       </c>
       <c r="B59" s="2" t="n">
-        <v>46030.20833333334</v>
+        <v>46114.95833333334</v>
       </c>
       <c r="C59" s="2" t="n">
-        <v>46031.95833333334</v>
+        <v>46115.33333333334</v>
       </c>
       <c r="D59" t="n">
-        <v>43</v>
+        <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>2.329966376477916</v>
+        <v>2.798742539278037</v>
       </c>
       <c r="F59" t="n">
-        <v>2.487220619812446</v>
+        <v>2.860378239024466</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -2213,29 +2213,29 @@
         </is>
       </c>
       <c r="H59" t="n">
-        <v>1.000390216394669</v>
+        <v>1.000170122637875</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ORP_1_2</t>
+          <t>ORP_1_1</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
-        <v>46033.75</v>
+        <v>46115.70833333334</v>
       </c>
       <c r="C60" s="2" t="n">
-        <v>46038.20833333334</v>
+        <v>46115.91666666666</v>
       </c>
       <c r="D60" t="n">
-        <v>108</v>
+        <v>6</v>
       </c>
       <c r="E60" t="n">
-        <v>2.476604834805639</v>
+        <v>2.82685896567884</v>
       </c>
       <c r="F60" t="n">
-        <v>2.499783378100052</v>
+        <v>2.865204925287654</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -2243,29 +2243,29 @@
         </is>
       </c>
       <c r="H60" t="n">
-        <v>1.100553793654593</v>
+        <v>1.005129204816508</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>ORP_1_2</t>
+          <t>ORP_1_1</t>
         </is>
       </c>
       <c r="B61" s="2" t="n">
-        <v>46063.875</v>
+        <v>46117.58333333334</v>
       </c>
       <c r="C61" s="2" t="n">
-        <v>46064.08333333334</v>
+        <v>46117.79166666666</v>
       </c>
       <c r="D61" t="n">
         <v>6</v>
       </c>
       <c r="E61" t="n">
-        <v>2.697815206233115</v>
+        <v>2.722453332391307</v>
       </c>
       <c r="F61" t="n">
-        <v>2.758551113549672</v>
+        <v>2.800563384417298</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
         </is>
       </c>
       <c r="H61" t="n">
-        <v>1.000034426564749</v>
+        <v>1.014371043248799</v>
       </c>
     </row>
     <row r="62">
@@ -2283,19 +2283,19 @@
         </is>
       </c>
       <c r="B62" s="2" t="n">
-        <v>46065.83333333334</v>
+        <v>46011.91666666666</v>
       </c>
       <c r="C62" s="2" t="n">
-        <v>46066.25</v>
+        <v>46012.29166666666</v>
       </c>
       <c r="D62" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>2.534730678598093</v>
+        <v>2.757967584852246</v>
       </c>
       <c r="F62" t="n">
-        <v>2.670238476054251</v>
+        <v>2.871753695513218</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -2303,7 +2303,7 @@
         </is>
       </c>
       <c r="H62" t="n">
-        <v>1.000390156597997</v>
+        <v>1.000000448472733</v>
       </c>
     </row>
     <row r="63">
@@ -2313,19 +2313,19 @@
         </is>
       </c>
       <c r="B63" s="2" t="n">
-        <v>46067.29166666666</v>
+        <v>46013.41666666666</v>
       </c>
       <c r="C63" s="2" t="n">
-        <v>46067.58333333334</v>
+        <v>46013.75</v>
       </c>
       <c r="D63" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E63" t="n">
-        <v>2.58962841072771</v>
+        <v>2.545127570053714</v>
       </c>
       <c r="F63" t="n">
-        <v>2.727744389683214</v>
+        <v>2.771131515972993</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -2333,7 +2333,7 @@
         </is>
       </c>
       <c r="H63" t="n">
-        <v>1.000097777091265</v>
+        <v>1.000017137212721</v>
       </c>
     </row>
     <row r="64">
@@ -2343,19 +2343,19 @@
         </is>
       </c>
       <c r="B64" s="2" t="n">
-        <v>46068.33333333334</v>
+        <v>46015.375</v>
       </c>
       <c r="C64" s="2" t="n">
-        <v>46068.625</v>
+        <v>46015.625</v>
       </c>
       <c r="D64" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E64" t="n">
-        <v>2.479357681581647</v>
+        <v>2.691704116627942</v>
       </c>
       <c r="F64" t="n">
-        <v>2.670418179514225</v>
+        <v>2.75093162892788</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -2363,7 +2363,7 @@
         </is>
       </c>
       <c r="H64" t="n">
-        <v>1.000625069863307</v>
+        <v>1.001564884736407</v>
       </c>
     </row>
     <row r="65">
@@ -2373,19 +2373,19 @@
         </is>
       </c>
       <c r="B65" s="2" t="n">
-        <v>46069.70833333334</v>
+        <v>46017.33333333334</v>
       </c>
       <c r="C65" s="2" t="n">
-        <v>46077.91666666666</v>
+        <v>46017.79166666666</v>
       </c>
       <c r="D65" t="n">
-        <v>198</v>
+        <v>12</v>
       </c>
       <c r="E65" t="n">
-        <v>2.413148214499939</v>
+        <v>2.387246484347651</v>
       </c>
       <c r="F65" t="n">
-        <v>2.501440487754722</v>
+        <v>2.586018094466748</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -2393,7 +2393,7 @@
         </is>
       </c>
       <c r="H65" t="n">
-        <v>1.000000010907038</v>
+        <v>1.000000351049599</v>
       </c>
     </row>
     <row r="66">
@@ -2403,13 +2403,13 @@
         </is>
       </c>
       <c r="B66" s="2" t="n">
-        <v>46078.41666666666</v>
+        <v>46018</v>
       </c>
       <c r="C66" s="2" t="n">
-        <v>46082.125</v>
+        <v>46028.25</v>
       </c>
       <c r="D66" t="n">
-        <v>90</v>
+        <v>247</v>
       </c>
       <c r="E66" t="n">
         <v>2.5</v>
@@ -2419,11 +2419,11 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_regime</t>
         </is>
       </c>
       <c r="H66" t="n">
-        <v>1.068234383831886</v>
+        <v>1.081134041730266</v>
       </c>
     </row>
     <row r="67">
@@ -2433,27 +2433,27 @@
         </is>
       </c>
       <c r="B67" s="2" t="n">
-        <v>46082.25</v>
+        <v>46030.20833333334</v>
       </c>
       <c r="C67" s="2" t="n">
-        <v>46089.25</v>
+        <v>46031.95833333334</v>
       </c>
       <c r="D67" t="n">
-        <v>169</v>
+        <v>43</v>
       </c>
       <c r="E67" t="n">
-        <v>2.5</v>
+        <v>2.329966376477916</v>
       </c>
       <c r="F67" t="n">
-        <v>2.5</v>
+        <v>2.487220619812446</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Q_regime</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H67" t="n">
-        <v>1.333577532071762</v>
+        <v>1.000390216394669</v>
       </c>
     </row>
     <row r="68">
@@ -2463,19 +2463,19 @@
         </is>
       </c>
       <c r="B68" s="2" t="n">
-        <v>46115</v>
+        <v>46033.75</v>
       </c>
       <c r="C68" s="2" t="n">
-        <v>46115.29166666666</v>
+        <v>46038.20833333334</v>
       </c>
       <c r="D68" t="n">
-        <v>8</v>
+        <v>108</v>
       </c>
       <c r="E68" t="n">
-        <v>2.481712743778947</v>
+        <v>2.476604834805639</v>
       </c>
       <c r="F68" t="n">
-        <v>2.645869648668306</v>
+        <v>2.499783378100052</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
@@ -2483,7 +2483,7 @@
         </is>
       </c>
       <c r="H68" t="n">
-        <v>1.102732574463459</v>
+        <v>1.100553793654593</v>
       </c>
     </row>
     <row r="69">
@@ -2493,19 +2493,19 @@
         </is>
       </c>
       <c r="B69" s="2" t="n">
-        <v>46117.58333333334</v>
+        <v>46063.875</v>
       </c>
       <c r="C69" s="2" t="n">
-        <v>46117.95833333334</v>
+        <v>46064.08333333334</v>
       </c>
       <c r="D69" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E69" t="n">
-        <v>2.5</v>
+        <v>2.697827570263692</v>
       </c>
       <c r="F69" t="n">
-        <v>2.620961897829237</v>
+        <v>2.759687927049036</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="H69" t="n">
-        <v>1.546691130829444</v>
+        <v>1.000058490844518</v>
       </c>
     </row>
     <row r="70">
@@ -2523,19 +2523,19 @@
         </is>
       </c>
       <c r="B70" s="2" t="n">
-        <v>46118.5</v>
+        <v>46065.83333333334</v>
       </c>
       <c r="C70" s="2" t="n">
-        <v>46122.45833333334</v>
+        <v>46066.25</v>
       </c>
       <c r="D70" t="n">
-        <v>96</v>
+        <v>11</v>
       </c>
       <c r="E70" t="n">
-        <v>2.426672063099368</v>
+        <v>2.534839148226271</v>
       </c>
       <c r="F70" t="n">
-        <v>2.498788344672366</v>
+        <v>2.672031339188797</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
@@ -2543,113 +2543,113 @@
         </is>
       </c>
       <c r="H70" t="n">
-        <v>1.016919746167972</v>
+        <v>1.000591289877526</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>ORP_1_3</t>
+          <t>ORP_1_2</t>
         </is>
       </c>
       <c r="B71" s="2" t="n">
-        <v>45944.5</v>
+        <v>46067.29166666666</v>
       </c>
       <c r="C71" s="2" t="n">
-        <v>45944.70833333334</v>
+        <v>46067.58333333334</v>
       </c>
       <c r="D71" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E71" t="n">
-        <v>2.359579249772268</v>
+        <v>2.592961524228548</v>
       </c>
       <c r="F71" t="n">
-        <v>2.540101005989568</v>
+        <v>2.729217713985539</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Q_step</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H71" t="n">
-        <v>1.239094636012759</v>
+        <v>1.000176110832394</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>ORP_1_3</t>
+          <t>ORP_1_2</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
-        <v>45945.25</v>
+        <v>46068.33333333334</v>
       </c>
       <c r="C72" s="2" t="n">
-        <v>45945.45833333334</v>
+        <v>46068.625</v>
       </c>
       <c r="D72" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E72" t="n">
-        <v>2.5</v>
+        <v>2.480221425257873</v>
       </c>
       <c r="F72" t="n">
-        <v>2.5</v>
+        <v>2.663636670467292</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Q_regime</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H72" t="n">
-        <v>1.961678843667339</v>
+        <v>1.001407905053316</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>ORP_1_3</t>
+          <t>ORP_1_2</t>
         </is>
       </c>
       <c r="B73" s="2" t="n">
-        <v>45946.5</v>
+        <v>46069.70833333334</v>
       </c>
       <c r="C73" s="2" t="n">
-        <v>45948.41666666666</v>
+        <v>46077.91666666666</v>
       </c>
       <c r="D73" t="n">
-        <v>47</v>
+        <v>198</v>
       </c>
       <c r="E73" t="n">
-        <v>2.5</v>
+        <v>2.413148214499939</v>
       </c>
       <c r="F73" t="n">
-        <v>2.5</v>
+        <v>2.501817813877794</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Q_regime</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H73" t="n">
-        <v>2.108098132368428</v>
+        <v>1.000000021182844</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>ORP_1_3</t>
+          <t>ORP_1_2</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
-        <v>45948.58333333334</v>
+        <v>46078.41666666666</v>
       </c>
       <c r="C74" s="2" t="n">
-        <v>45949.5</v>
+        <v>46082.125</v>
       </c>
       <c r="D74" t="n">
-        <v>23</v>
+        <v>90</v>
       </c>
       <c r="E74" t="n">
         <v>2.5</v>
@@ -2659,63 +2659,63 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Q_step</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H74" t="n">
-        <v>3.133136153004526</v>
+        <v>1.068234383831886</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>ORP_1_3</t>
+          <t>ORP_1_2</t>
         </is>
       </c>
       <c r="B75" s="2" t="n">
-        <v>45985.875</v>
+        <v>46082.25</v>
       </c>
       <c r="C75" s="2" t="n">
-        <v>45986.08333333334</v>
+        <v>46089.25</v>
       </c>
       <c r="D75" t="n">
-        <v>6</v>
+        <v>169</v>
       </c>
       <c r="E75" t="n">
-        <v>2.532284377008832</v>
+        <v>2.5</v>
       </c>
       <c r="F75" t="n">
-        <v>2.702907353326314</v>
+        <v>2.5</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Q_step</t>
+          <t>Q_regime</t>
         </is>
       </c>
       <c r="H75" t="n">
-        <v>1.156662891187058</v>
+        <v>1.333577532071762</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>ORP_2_1</t>
+          <t>ORP_1_2</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
-        <v>45912.66666666666</v>
+        <v>46115</v>
       </c>
       <c r="C76" s="2" t="n">
-        <v>45912.91666666666</v>
+        <v>46115.29166666666</v>
       </c>
       <c r="D76" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E76" t="n">
-        <v>2.916844687683574</v>
+        <v>2.481712743778947</v>
       </c>
       <c r="F76" t="n">
-        <v>2.959759002487399</v>
+        <v>2.645869648668306</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
@@ -2723,29 +2723,29 @@
         </is>
       </c>
       <c r="H76" t="n">
-        <v>1.000377368846203</v>
+        <v>1.102732574463459</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>ORP_2_1</t>
+          <t>ORP_1_2</t>
         </is>
       </c>
       <c r="B77" s="2" t="n">
-        <v>45913.58333333334</v>
+        <v>46117.58333333334</v>
       </c>
       <c r="C77" s="2" t="n">
-        <v>45914</v>
+        <v>46117.95833333334</v>
       </c>
       <c r="D77" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>2.815254810454179</v>
+        <v>2.5</v>
       </c>
       <c r="F77" t="n">
-        <v>2.875642517265083</v>
+        <v>2.620961897829237</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -2753,29 +2753,29 @@
         </is>
       </c>
       <c r="H77" t="n">
-        <v>1.001948134034438</v>
+        <v>1.546691130829444</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>ORP_2_1</t>
+          <t>ORP_1_2</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
-        <v>46103.54166666666</v>
+        <v>46118.5</v>
       </c>
       <c r="C78" s="2" t="n">
-        <v>46103.75</v>
+        <v>46122.45833333334</v>
       </c>
       <c r="D78" t="n">
-        <v>6</v>
+        <v>96</v>
       </c>
       <c r="E78" t="n">
-        <v>2.924219619702625</v>
+        <v>2.426672063099368</v>
       </c>
       <c r="F78" t="n">
-        <v>2.945838210010882</v>
+        <v>2.498788344672366</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -2783,53 +2783,53 @@
         </is>
       </c>
       <c r="H78" t="n">
-        <v>1.000677252565855</v>
+        <v>1.016919746167972</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>ORP_2_2</t>
+          <t>ORP_1_3</t>
         </is>
       </c>
       <c r="B79" s="2" t="n">
-        <v>46018.75</v>
+        <v>45944.5</v>
       </c>
       <c r="C79" s="2" t="n">
-        <v>46019</v>
+        <v>45944.70833333334</v>
       </c>
       <c r="D79" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E79" t="n">
-        <v>2.734094841154886</v>
+        <v>2.359579249772268</v>
       </c>
       <c r="F79" t="n">
-        <v>2.860673160381919</v>
+        <v>2.540101005989568</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_step</t>
         </is>
       </c>
       <c r="H79" t="n">
-        <v>1.031984641824361</v>
+        <v>1.239094636012759</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>ORP_2_2</t>
+          <t>ORP_1_3</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
-        <v>46036.75</v>
+        <v>45945.25</v>
       </c>
       <c r="C80" s="2" t="n">
-        <v>46037.45833333334</v>
+        <v>45945.45833333334</v>
       </c>
       <c r="D80" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="E80" t="n">
         <v>2.5</v>
@@ -2843,66 +2843,276 @@
         </is>
       </c>
       <c r="H80" t="n">
-        <v>1.922445730625928</v>
+        <v>1.961678843667339</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>ORP_2_2</t>
+          <t>ORP_1_3</t>
         </is>
       </c>
       <c r="B81" s="2" t="n">
-        <v>46080.58333333334</v>
+        <v>45946.5</v>
       </c>
       <c r="C81" s="2" t="n">
-        <v>46080.79166666666</v>
+        <v>45948.41666666666</v>
       </c>
       <c r="D81" t="n">
-        <v>6</v>
+        <v>47</v>
       </c>
       <c r="E81" t="n">
-        <v>2.81960042268659</v>
+        <v>2.5</v>
       </c>
       <c r="F81" t="n">
-        <v>2.893198009776475</v>
+        <v>2.5</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_regime</t>
         </is>
       </c>
       <c r="H81" t="n">
-        <v>1.005173111560453</v>
+        <v>2.108098132368428</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
+          <t>ORP_1_3</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="n">
+        <v>45948.58333333334</v>
+      </c>
+      <c r="C82" s="2" t="n">
+        <v>45949.5</v>
+      </c>
+      <c r="D82" t="n">
+        <v>23</v>
+      </c>
+      <c r="E82" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F82" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Q_step</t>
+        </is>
+      </c>
+      <c r="H82" t="n">
+        <v>3.133136153004526</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>ORP_1_3</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="n">
+        <v>45985.875</v>
+      </c>
+      <c r="C83" s="2" t="n">
+        <v>45986.08333333334</v>
+      </c>
+      <c r="D83" t="n">
+        <v>6</v>
+      </c>
+      <c r="E83" t="n">
+        <v>2.532284377008832</v>
+      </c>
+      <c r="F83" t="n">
+        <v>2.702907353326314</v>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Q_step</t>
+        </is>
+      </c>
+      <c r="H83" t="n">
+        <v>1.156662891187058</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>ORP_2_1</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="n">
+        <v>45912.66666666666</v>
+      </c>
+      <c r="C84" s="2" t="n">
+        <v>45912.91666666666</v>
+      </c>
+      <c r="D84" t="n">
+        <v>7</v>
+      </c>
+      <c r="E84" t="n">
+        <v>2.916749424863698</v>
+      </c>
+      <c r="F84" t="n">
+        <v>2.958434285225183</v>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Q_drift</t>
+        </is>
+      </c>
+      <c r="H84" t="n">
+        <v>1.000403757743586</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>ORP_2_1</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="n">
+        <v>45913.58333333334</v>
+      </c>
+      <c r="C85" s="2" t="n">
+        <v>45914</v>
+      </c>
+      <c r="D85" t="n">
+        <v>11</v>
+      </c>
+      <c r="E85" t="n">
+        <v>2.813665244581917</v>
+      </c>
+      <c r="F85" t="n">
+        <v>2.870842326941625</v>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Q_drift</t>
+        </is>
+      </c>
+      <c r="H85" t="n">
+        <v>1.001934196184946</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
           <t>ORP_2_2</t>
         </is>
       </c>
-      <c r="B82" s="2" t="n">
+      <c r="B86" s="2" t="n">
+        <v>46018.75</v>
+      </c>
+      <c r="C86" s="2" t="n">
+        <v>46019</v>
+      </c>
+      <c r="D86" t="n">
+        <v>7</v>
+      </c>
+      <c r="E86" t="n">
+        <v>2.734094841154886</v>
+      </c>
+      <c r="F86" t="n">
+        <v>2.860673160381919</v>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Q_drift</t>
+        </is>
+      </c>
+      <c r="H86" t="n">
+        <v>1.031984641824361</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>ORP_2_2</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="n">
+        <v>46036.75</v>
+      </c>
+      <c r="C87" s="2" t="n">
+        <v>46037.45833333334</v>
+      </c>
+      <c r="D87" t="n">
+        <v>18</v>
+      </c>
+      <c r="E87" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F87" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Q_regime</t>
+        </is>
+      </c>
+      <c r="H87" t="n">
+        <v>1.922445730625928</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>ORP_2_2</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="n">
+        <v>46080.58333333334</v>
+      </c>
+      <c r="C88" s="2" t="n">
+        <v>46080.79166666666</v>
+      </c>
+      <c r="D88" t="n">
+        <v>6</v>
+      </c>
+      <c r="E88" t="n">
+        <v>2.81960042268659</v>
+      </c>
+      <c r="F88" t="n">
+        <v>2.893198009776475</v>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Q_drift</t>
+        </is>
+      </c>
+      <c r="H88" t="n">
+        <v>1.005173111560453</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>ORP_2_2</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="n">
         <v>46119</v>
       </c>
-      <c r="C82" s="2" t="n">
+      <c r="C89" s="2" t="n">
         <v>46122.45833333334</v>
       </c>
-      <c r="D82" t="n">
+      <c r="D89" t="n">
         <v>84</v>
       </c>
-      <c r="E82" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="F82" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="G82" t="inlineStr">
+      <c r="E89" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F89" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G89" t="inlineStr">
         <is>
           <t>Q_regime</t>
         </is>
       </c>
-      <c r="H82" t="n">
+      <c r="H89" t="n">
         <v>1.160462951377068</v>
       </c>
     </row>
@@ -2917,7 +3127,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H63"/>
+  <dimension ref="A1:H62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2978,10 +3188,10 @@
         <v>7</v>
       </c>
       <c r="E2" t="n">
-        <v>2.776674147507447</v>
+        <v>2.778023496646145</v>
       </c>
       <c r="F2" t="n">
-        <v>2.84874268532911</v>
+        <v>2.849906663019707</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -2989,7 +3199,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>1.000005614214015</v>
+        <v>1.000005525074796</v>
       </c>
     </row>
     <row r="3">
@@ -3008,10 +3218,10 @@
         <v>6</v>
       </c>
       <c r="E3" t="n">
-        <v>2.82166051957243</v>
+        <v>2.817097209666348</v>
       </c>
       <c r="F3" t="n">
-        <v>2.955211575393891</v>
+        <v>2.950866201389108</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -3019,7 +3229,7 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>1.084277888278427</v>
+        <v>1.078295198584504</v>
       </c>
     </row>
     <row r="4">
@@ -3359,19 +3569,19 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>45923.29166666666</v>
+        <v>46109.875</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>45927.20833333334</v>
+        <v>46110.20833333334</v>
       </c>
       <c r="D15" t="n">
-        <v>95</v>
+        <v>9</v>
       </c>
       <c r="E15" t="n">
         <v>2.5</v>
       </c>
       <c r="F15" t="n">
-        <v>2.504750233674428</v>
+        <v>2.631945023120458</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -3379,7 +3589,7 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>1.007870807954773</v>
+        <v>1.177011940529713</v>
       </c>
     </row>
     <row r="16">
@@ -3389,19 +3599,19 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>45914.25</v>
+        <v>45923.29166666666</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>45923.08333333334</v>
+        <v>45927.20833333334</v>
       </c>
       <c r="D16" t="n">
-        <v>213</v>
+        <v>95</v>
       </c>
       <c r="E16" t="n">
         <v>2.5</v>
       </c>
       <c r="F16" t="n">
-        <v>2.5</v>
+        <v>2.504750233674428</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -3409,7 +3619,7 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>1.000027425415349</v>
+        <v>1.007870807954773</v>
       </c>
     </row>
     <row r="17">
@@ -3419,19 +3629,19 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>45927.29166666666</v>
+        <v>45914.25</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>45929.08333333334</v>
+        <v>45923.08333333334</v>
       </c>
       <c r="D17" t="n">
-        <v>44</v>
+        <v>213</v>
       </c>
       <c r="E17" t="n">
         <v>2.5</v>
       </c>
       <c r="F17" t="n">
-        <v>2.513093523236048</v>
+        <v>2.5</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -3439,7 +3649,7 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>1.000024569032804</v>
+        <v>1.000027425415349</v>
       </c>
     </row>
     <row r="18">
@@ -3449,19 +3659,19 @@
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>45929.29166666666</v>
+        <v>45927.29166666666</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>45931.20833333334</v>
+        <v>45929.08333333334</v>
       </c>
       <c r="D18" t="n">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="E18" t="n">
         <v>2.5</v>
       </c>
       <c r="F18" t="n">
-        <v>2.516133291750057</v>
+        <v>2.513093523236048</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -3469,7 +3679,7 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>1.005320194675679</v>
+        <v>1.000024569032804</v>
       </c>
     </row>
     <row r="19">
@@ -3509,19 +3719,19 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>46109.875</v>
+        <v>45929.29166666666</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>46110.20833333334</v>
+        <v>45931.20833333334</v>
       </c>
       <c r="D20" t="n">
-        <v>9</v>
+        <v>47</v>
       </c>
       <c r="E20" t="n">
         <v>2.5</v>
       </c>
       <c r="F20" t="n">
-        <v>2.631945023120458</v>
+        <v>2.516133291750057</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -3529,7 +3739,7 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>1.177011940529713</v>
+        <v>1.005320194675679</v>
       </c>
     </row>
     <row r="21">
@@ -3569,27 +3779,27 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>46102.91666666666</v>
+        <v>46102.875</v>
       </c>
       <c r="C22" s="2" t="n">
         <v>46103.33333333334</v>
       </c>
       <c r="D22" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E22" t="n">
         <v>2</v>
       </c>
       <c r="F22" t="n">
-        <v>2.081402219039941</v>
+        <v>2.114764389726374</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Q_freeze</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H22" t="n">
-        <v>1.226970741004972</v>
+        <v>1.000081729568714</v>
       </c>
     </row>
     <row r="23">
@@ -3599,19 +3809,19 @@
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>46011.91666666666</v>
+        <v>45998.66666666666</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>46012.125</v>
+        <v>45998.875</v>
       </c>
       <c r="D23" t="n">
         <v>6</v>
       </c>
       <c r="E23" t="n">
-        <v>2.400909013242728</v>
+        <v>2.211936251292717</v>
       </c>
       <c r="F23" t="n">
-        <v>2.583739404377635</v>
+        <v>2.479658830044532</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -3619,7 +3829,7 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>1.000005203420343</v>
+        <v>1.0189217456638</v>
       </c>
     </row>
     <row r="24">
@@ -3629,19 +3839,19 @@
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>45984.45833333334</v>
+        <v>46011.91666666666</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>45984.91666666666</v>
+        <v>46012.20833333334</v>
       </c>
       <c r="D24" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E24" t="n">
-        <v>2.447921818153538</v>
+        <v>2.392805004675806</v>
       </c>
       <c r="F24" t="n">
-        <v>2.717737062928489</v>
+        <v>2.596736357047955</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -3649,7 +3859,7 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>1.00000065855702</v>
+        <v>1.000015078979207</v>
       </c>
     </row>
     <row r="25">
@@ -3659,19 +3869,19 @@
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>46013.66666666666</v>
+        <v>45984.45833333334</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>46014.20833333334</v>
+        <v>45984.91666666666</v>
       </c>
       <c r="D25" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E25" t="n">
-        <v>2.451291985467262</v>
+        <v>2.447935866890584</v>
       </c>
       <c r="F25" t="n">
-        <v>2.67249520178254</v>
+        <v>2.718102655457825</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -3679,7 +3889,7 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>1.000000000738104</v>
+        <v>1.000001103825005</v>
       </c>
     </row>
     <row r="26">
@@ -3689,27 +3899,27 @@
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>45985</v>
+        <v>46013.66666666666</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>45985.54166666666</v>
+        <v>46014.16666666666</v>
       </c>
       <c r="D26" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E26" t="n">
-        <v>2.550175579847397</v>
+        <v>2.451277291557278</v>
       </c>
       <c r="F26" t="n">
-        <v>2.71946138852274</v>
+        <v>2.664274531537799</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Q_step</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H26" t="n">
-        <v>1.156662891187058</v>
+        <v>1.000000000141117</v>
       </c>
     </row>
     <row r="27">
@@ -3719,19 +3929,19 @@
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>46011.45833333334</v>
+        <v>46068.75</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>46011.83333333334</v>
+        <v>46069.125</v>
       </c>
       <c r="D27" t="n">
         <v>10</v>
       </c>
       <c r="E27" t="n">
-        <v>2.567188046035585</v>
+        <v>2.534498966663721</v>
       </c>
       <c r="F27" t="n">
-        <v>2.646585973935476</v>
+        <v>2.670607565166778</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -3739,7 +3949,7 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>1.000000028806149</v>
+        <v>1.029970506055951</v>
       </c>
     </row>
     <row r="28">
@@ -3749,27 +3959,27 @@
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>45982.66666666666</v>
+        <v>45985</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>45983.45833333334</v>
+        <v>45985.54166666666</v>
       </c>
       <c r="D28" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="E28" t="n">
-        <v>2.590874993410552</v>
+        <v>2.550175579847397</v>
       </c>
       <c r="F28" t="n">
-        <v>2.842002306336331</v>
+        <v>2.71946138852274</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_step</t>
         </is>
       </c>
       <c r="H28" t="n">
-        <v>1.000001443244321</v>
+        <v>1.156662891187058</v>
       </c>
     </row>
     <row r="29">
@@ -3779,19 +3989,19 @@
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>45920.75</v>
+        <v>46029.625</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>45921.04166666666</v>
+        <v>46029.875</v>
       </c>
       <c r="D29" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E29" t="n">
-        <v>2.631283258737578</v>
+        <v>2.567062194481823</v>
       </c>
       <c r="F29" t="n">
-        <v>2.86650035514931</v>
+        <v>2.755760587104711</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -3799,7 +4009,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>1.000395008168533</v>
+        <v>1.001531969385012</v>
       </c>
     </row>
     <row r="30">
@@ -3809,27 +4019,27 @@
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>46014.45833333334</v>
+        <v>46011.5</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>46014.66666666666</v>
+        <v>46011.83333333334</v>
       </c>
       <c r="D30" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E30" t="n">
-        <v>2.776726839400139</v>
+        <v>2.567194367272065</v>
       </c>
       <c r="F30" t="n">
-        <v>2.819586287662029</v>
+        <v>2.64530938286319</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Q_step</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H30" t="n">
-        <v>1.535711553296295</v>
+        <v>1.000000067627254</v>
       </c>
     </row>
     <row r="31">
@@ -3839,19 +4049,19 @@
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>45919.66666666666</v>
+        <v>46077.70833333334</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>45920.04166666666</v>
+        <v>46078</v>
       </c>
       <c r="D31" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E31" t="n">
-        <v>2.807613851151439</v>
+        <v>2.588607853112589</v>
       </c>
       <c r="F31" t="n">
-        <v>2.862055297206406</v>
+        <v>2.84003479810486</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -3859,7 +4069,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>1.00472076843603</v>
+        <v>1.03956381193685</v>
       </c>
     </row>
     <row r="32">
@@ -4208,10 +4418,10 @@
         <v>12</v>
       </c>
       <c r="E43" t="n">
-        <v>2.38724600616407</v>
+        <v>2.387246484347651</v>
       </c>
       <c r="F43" t="n">
-        <v>2.584654464869179</v>
+        <v>2.586018094466748</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -4219,7 +4429,7 @@
         </is>
       </c>
       <c r="H43" t="n">
-        <v>1.000000453251144</v>
+        <v>1.000000351049599</v>
       </c>
     </row>
     <row r="44">
@@ -4241,7 +4451,7 @@
         <v>2.413148214499939</v>
       </c>
       <c r="F44" t="n">
-        <v>2.501440487754722</v>
+        <v>2.501817813877794</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -4249,7 +4459,7 @@
         </is>
       </c>
       <c r="H44" t="n">
-        <v>1.000000010907038</v>
+        <v>1.000000021182844</v>
       </c>
     </row>
     <row r="45">
@@ -4328,10 +4538,10 @@
         <v>8</v>
       </c>
       <c r="E47" t="n">
-        <v>2.479357681581647</v>
+        <v>2.480221425257873</v>
       </c>
       <c r="F47" t="n">
-        <v>2.670418179514225</v>
+        <v>2.663636670467292</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -4339,7 +4549,7 @@
         </is>
       </c>
       <c r="H47" t="n">
-        <v>1.000625069863307</v>
+        <v>1.001407905053316</v>
       </c>
     </row>
     <row r="48">
@@ -4382,10 +4592,10 @@
         <v>46018</v>
       </c>
       <c r="C49" s="2" t="n">
-        <v>46028.29166666666</v>
+        <v>46028.25</v>
       </c>
       <c r="D49" t="n">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E49" t="n">
         <v>2.5</v>
@@ -4628,10 +4838,10 @@
         <v>11</v>
       </c>
       <c r="E57" t="n">
-        <v>2.815254810454179</v>
+        <v>2.813665244581917</v>
       </c>
       <c r="F57" t="n">
-        <v>2.875642517265083</v>
+        <v>2.870842326941625</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -4639,7 +4849,7 @@
         </is>
       </c>
       <c r="H57" t="n">
-        <v>1.001948134034438</v>
+        <v>1.001934196184946</v>
       </c>
     </row>
     <row r="58">
@@ -4658,10 +4868,10 @@
         <v>7</v>
       </c>
       <c r="E58" t="n">
-        <v>2.916844687683574</v>
+        <v>2.916749424863698</v>
       </c>
       <c r="F58" t="n">
-        <v>2.959759002487399</v>
+        <v>2.958434285225183</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -4669,37 +4879,37 @@
         </is>
       </c>
       <c r="H58" t="n">
-        <v>1.000377368846203</v>
+        <v>1.000403757743586</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>ORP_2_1</t>
+          <t>ORP_2_2</t>
         </is>
       </c>
       <c r="B59" s="2" t="n">
-        <v>46103.54166666666</v>
+        <v>46119</v>
       </c>
       <c r="C59" s="2" t="n">
-        <v>46103.75</v>
+        <v>46122.45833333334</v>
       </c>
       <c r="D59" t="n">
-        <v>6</v>
+        <v>84</v>
       </c>
       <c r="E59" t="n">
-        <v>2.924219619702625</v>
+        <v>2.5</v>
       </c>
       <c r="F59" t="n">
-        <v>2.945838210010882</v>
+        <v>2.5</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_regime</t>
         </is>
       </c>
       <c r="H59" t="n">
-        <v>1.000677252565855</v>
+        <v>1.160462951377068</v>
       </c>
     </row>
     <row r="60">
@@ -4739,27 +4949,27 @@
         </is>
       </c>
       <c r="B61" s="2" t="n">
-        <v>46119</v>
+        <v>46018.75</v>
       </c>
       <c r="C61" s="2" t="n">
-        <v>46122.45833333334</v>
+        <v>46019</v>
       </c>
       <c r="D61" t="n">
-        <v>84</v>
+        <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>2.5</v>
+        <v>2.734094841154886</v>
       </c>
       <c r="F61" t="n">
-        <v>2.5</v>
+        <v>2.860673160381919</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Q_regime</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H61" t="n">
-        <v>1.160462951377068</v>
+        <v>1.031984641824361</v>
       </c>
     </row>
     <row r="62">
@@ -4769,19 +4979,19 @@
         </is>
       </c>
       <c r="B62" s="2" t="n">
-        <v>46018.75</v>
+        <v>46080.58333333334</v>
       </c>
       <c r="C62" s="2" t="n">
-        <v>46019</v>
+        <v>46080.79166666666</v>
       </c>
       <c r="D62" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E62" t="n">
-        <v>2.734094841154886</v>
+        <v>2.81960042268659</v>
       </c>
       <c r="F62" t="n">
-        <v>2.860673160381919</v>
+        <v>2.893198009776475</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -4789,36 +4999,6 @@
         </is>
       </c>
       <c r="H62" t="n">
-        <v>1.031984641824361</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>ORP_2_2</t>
-        </is>
-      </c>
-      <c r="B63" s="2" t="n">
-        <v>46080.58333333334</v>
-      </c>
-      <c r="C63" s="2" t="n">
-        <v>46080.79166666666</v>
-      </c>
-      <c r="D63" t="n">
-        <v>6</v>
-      </c>
-      <c r="E63" t="n">
-        <v>2.81960042268659</v>
-      </c>
-      <c r="F63" t="n">
-        <v>2.893198009776475</v>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>Q_drift</t>
-        </is>
-      </c>
-      <c r="H63" t="n">
         <v>1.005173111560453</v>
       </c>
     </row>
@@ -4881,7 +5061,7 @@
         <v>13</v>
       </c>
       <c r="E2" t="n">
-        <v>2.799167333539939</v>
+        <v>2.797560353156246</v>
       </c>
     </row>
     <row r="3">
@@ -5064,13 +5244,13 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="D11" t="n">
-        <v>92</v>
+        <v>159</v>
       </c>
       <c r="E11" t="n">
-        <v>2.615200703095924</v>
+        <v>2.560832894283463</v>
       </c>
     </row>
     <row r="12">
@@ -5081,17 +5261,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Q_freeze</t>
+          <t>Q_spike</t>
         </is>
       </c>
       <c r="C12" t="n">
         <v>1</v>
       </c>
       <c r="D12" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E12" t="n">
-        <v>2</v>
+        <v>2.682590823715822</v>
       </c>
     </row>
     <row r="13">
@@ -5154,7 +5334,7 @@
         <v>624</v>
       </c>
       <c r="E15" t="n">
-        <v>2.520759942999768</v>
+        <v>2.521066643767983</v>
       </c>
     </row>
     <row r="16">
@@ -5172,7 +5352,7 @@
         <v>2</v>
       </c>
       <c r="D16" t="n">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="E16" t="n">
         <v>2.5</v>
@@ -5232,13 +5412,13 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D19" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="E19" t="n">
-        <v>2.885439705946792</v>
+        <v>2.865207334722808</v>
       </c>
     </row>
     <row r="20">

</xml_diff>

<commit_message>
Validate D1 DO2_4 PLS peer admission
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D1 Sensor health/outputs/data/D1_event_windows.xlsx
+++ b/Project 1 Data Quality Assessment/D1 Sensor health/outputs/data/D1_event_windows.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H89"/>
+  <dimension ref="A1:H82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1302,10 +1302,10 @@
         <v>6</v>
       </c>
       <c r="E29" t="n">
-        <v>2.825158860728377</v>
+        <v>2.829468115317858</v>
       </c>
       <c r="F29" t="n">
-        <v>2.879490557669677</v>
+        <v>2.887947844078032</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -1313,7 +1313,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>1.006655537563976</v>
+        <v>1.0157276524892</v>
       </c>
     </row>
     <row r="30">
@@ -1323,19 +1323,19 @@
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>45917.20833333334</v>
+        <v>45920.75</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>45917.41666666666</v>
+        <v>45921</v>
       </c>
       <c r="D30" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E30" t="n">
-        <v>2.809293725156838</v>
+        <v>2.645057429847372</v>
       </c>
       <c r="F30" t="n">
-        <v>2.853676095959244</v>
+        <v>2.860199471141084</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1343,7 +1343,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>1.000680342465465</v>
+        <v>1.008206399446979</v>
       </c>
     </row>
     <row r="31">
@@ -1353,19 +1353,19 @@
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>45919.66666666666</v>
+        <v>45952</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>45920.04166666666</v>
+        <v>45952.29166666666</v>
       </c>
       <c r="D31" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E31" t="n">
-        <v>2.810519000303214</v>
+        <v>2.711356801800613</v>
       </c>
       <c r="F31" t="n">
-        <v>2.853831015240609</v>
+        <v>2.874758353593821</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>1.005044614206155</v>
+        <v>1.002966988143756</v>
       </c>
     </row>
     <row r="32">
@@ -1383,19 +1383,19 @@
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>45920.75</v>
+        <v>45982.66666666666</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>45921.04166666666</v>
+        <v>45983.41666666666</v>
       </c>
       <c r="D32" t="n">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="E32" t="n">
-        <v>2.631677867231224</v>
+        <v>2.593419013399966</v>
       </c>
       <c r="F32" t="n">
-        <v>2.867962299653354</v>
+        <v>2.829096550849842</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -1403,7 +1403,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>1.002561889542912</v>
+        <v>1.000004287752132</v>
       </c>
     </row>
     <row r="33">
@@ -1413,19 +1413,19 @@
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>45952</v>
+        <v>45984.45833333334</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>45952.29166666666</v>
+        <v>45984.91666666666</v>
       </c>
       <c r="D33" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E33" t="n">
-        <v>2.721496201402909</v>
+        <v>2.44799296816425</v>
       </c>
       <c r="F33" t="n">
-        <v>2.868353618291169</v>
+        <v>2.717725229822283</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -1433,7 +1433,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>1.002264254450091</v>
+        <v>1.000001210556082</v>
       </c>
     </row>
     <row r="34">
@@ -1443,27 +1443,27 @@
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>45982.625</v>
+        <v>45985</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>45983.41666666666</v>
+        <v>45985.54166666666</v>
       </c>
       <c r="D34" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="E34" t="n">
-        <v>2.593590713815669</v>
+        <v>2.550175579847397</v>
       </c>
       <c r="F34" t="n">
-        <v>2.824028653460144</v>
+        <v>2.71946138852274</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_step</t>
         </is>
       </c>
       <c r="H34" t="n">
-        <v>1.000004535023473</v>
+        <v>1.156662891187058</v>
       </c>
     </row>
     <row r="35">
@@ -1473,19 +1473,19 @@
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>45984.45833333334</v>
+        <v>46011.5</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>45984.91666666666</v>
+        <v>46011.83333333334</v>
       </c>
       <c r="D35" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E35" t="n">
-        <v>2.447935866890584</v>
+        <v>2.567221759903792</v>
       </c>
       <c r="F35" t="n">
-        <v>2.718102655457825</v>
+        <v>2.641917370543523</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -1493,7 +1493,7 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>1.000001103825005</v>
+        <v>1.000000061891391</v>
       </c>
     </row>
     <row r="36">
@@ -1503,27 +1503,27 @@
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>45985</v>
+        <v>46011.91666666666</v>
       </c>
       <c r="C36" s="2" t="n">
-        <v>45985.54166666666</v>
+        <v>46012.16666666666</v>
       </c>
       <c r="D36" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E36" t="n">
-        <v>2.550175579847397</v>
+        <v>2.396590681906827</v>
       </c>
       <c r="F36" t="n">
-        <v>2.71946138852274</v>
+        <v>2.583110821007263</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Q_step</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H36" t="n">
-        <v>1.156662891187058</v>
+        <v>1.000022499433851</v>
       </c>
     </row>
     <row r="37">
@@ -1533,19 +1533,19 @@
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>45998.66666666666</v>
+        <v>46013.66666666666</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>45998.875</v>
+        <v>46014.16666666666</v>
       </c>
       <c r="D37" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="E37" t="n">
-        <v>2.211936251292717</v>
+        <v>2.451283473014483</v>
       </c>
       <c r="F37" t="n">
-        <v>2.479658830044532</v>
+        <v>2.664910159560438</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -1553,7 +1553,7 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>1.0189217456638</v>
+        <v>1.000000001127826</v>
       </c>
     </row>
     <row r="38">
@@ -1563,27 +1563,27 @@
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>46011.5</v>
+        <v>46014.45833333334</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>46011.83333333334</v>
+        <v>46014.66666666666</v>
       </c>
       <c r="D38" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E38" t="n">
-        <v>2.567194367272065</v>
+        <v>2.776726839400139</v>
       </c>
       <c r="F38" t="n">
-        <v>2.64530938286319</v>
+        <v>2.819586287662029</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_step</t>
         </is>
       </c>
       <c r="H38" t="n">
-        <v>1.000000067627254</v>
+        <v>1.535711553296295</v>
       </c>
     </row>
     <row r="39">
@@ -1593,19 +1593,19 @@
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>46011.91666666666</v>
+        <v>46029.66666666666</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>46012.20833333334</v>
+        <v>46029.875</v>
       </c>
       <c r="D39" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E39" t="n">
-        <v>2.392805004675806</v>
+        <v>2.650301756052542</v>
       </c>
       <c r="F39" t="n">
-        <v>2.596736357047955</v>
+        <v>2.783738827060561</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -1613,7 +1613,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>1.000015078979207</v>
+        <v>1.003314581123384</v>
       </c>
     </row>
     <row r="40">
@@ -1623,19 +1623,19 @@
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>46013.66666666666</v>
+        <v>46102.875</v>
       </c>
       <c r="C40" s="2" t="n">
-        <v>46014.16666666666</v>
+        <v>46103.33333333334</v>
       </c>
       <c r="D40" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E40" t="n">
-        <v>2.451277291557278</v>
+        <v>2</v>
       </c>
       <c r="F40" t="n">
-        <v>2.664274531537799</v>
+        <v>2.117137735246667</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -1643,7 +1643,7 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>1.000000000141117</v>
+        <v>1.011071265909375</v>
       </c>
     </row>
     <row r="41">
@@ -1653,49 +1653,49 @@
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>46014.45833333334</v>
+        <v>46103.75</v>
       </c>
       <c r="C41" s="2" t="n">
-        <v>46014.66666666666</v>
+        <v>46104.08333333334</v>
       </c>
       <c r="D41" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E41" t="n">
-        <v>2.776726839400139</v>
+        <v>2.701271638760034</v>
       </c>
       <c r="F41" t="n">
-        <v>2.819586287662029</v>
+        <v>2.829865795819057</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Q_step</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H41" t="n">
-        <v>1.535711553296295</v>
+        <v>1.027031614956905</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>DO_2_4</t>
+          <t>ORP_1_1</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>46029.625</v>
+        <v>45920.16666666666</v>
       </c>
       <c r="C42" s="2" t="n">
-        <v>46029.875</v>
+        <v>45920.375</v>
       </c>
       <c r="D42" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E42" t="n">
-        <v>2.567062194481823</v>
+        <v>2.757376328495986</v>
       </c>
       <c r="F42" t="n">
-        <v>2.755760587104711</v>
+        <v>2.879726012342237</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -1703,59 +1703,59 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>1.001531969385012</v>
+        <v>1.000007312976706</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>DO_2_4</t>
+          <t>ORP_1_1</t>
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>46064.29166666666</v>
+        <v>45972.875</v>
       </c>
       <c r="C43" s="2" t="n">
-        <v>46064.5</v>
+        <v>45973.125</v>
       </c>
       <c r="D43" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E43" t="n">
-        <v>2.682590823715822</v>
+        <v>2.809682021993101</v>
       </c>
       <c r="F43" t="n">
-        <v>2.766922847811539</v>
+        <v>2.874583149247187</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Q_spike</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H43" t="n">
-        <v>1</v>
+        <v>1.000251210791262</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>DO_2_4</t>
+          <t>ORP_1_1</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>46068.75</v>
+        <v>46031.41666666666</v>
       </c>
       <c r="C44" s="2" t="n">
-        <v>46069.125</v>
+        <v>46031.625</v>
       </c>
       <c r="D44" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E44" t="n">
-        <v>2.534498966663721</v>
+        <v>2.834374417406643</v>
       </c>
       <c r="F44" t="n">
-        <v>2.670607565166778</v>
+        <v>2.888146187617946</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -1763,29 +1763,29 @@
         </is>
       </c>
       <c r="H44" t="n">
-        <v>1.029970506055951</v>
+        <v>1.012556226373021</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>DO_2_4</t>
+          <t>ORP_1_1</t>
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>46070.29166666666</v>
+        <v>46069.70833333334</v>
       </c>
       <c r="C45" s="2" t="n">
-        <v>46070.5</v>
+        <v>46070.08333333334</v>
       </c>
       <c r="D45" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>2.703520320400192</v>
+        <v>2.896610077643929</v>
       </c>
       <c r="F45" t="n">
-        <v>2.844309062842978</v>
+        <v>2.925288845222536</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -1793,29 +1793,29 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>1.230426783607971</v>
+        <v>1.000175276400918</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>DO_2_4</t>
+          <t>ORP_1_1</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>46077.70833333334</v>
+        <v>46070.66666666666</v>
       </c>
       <c r="C46" s="2" t="n">
-        <v>46078</v>
+        <v>46070.875</v>
       </c>
       <c r="D46" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E46" t="n">
-        <v>2.588607853112589</v>
+        <v>2.862447879436455</v>
       </c>
       <c r="F46" t="n">
-        <v>2.84003479810486</v>
+        <v>2.904058513690617</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -1823,29 +1823,29 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>1.03956381193685</v>
+        <v>1.000000824987803</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>DO_2_4</t>
+          <t>ORP_1_1</t>
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>46102.875</v>
+        <v>46071.16666666666</v>
       </c>
       <c r="C47" s="2" t="n">
-        <v>46103.33333333334</v>
+        <v>46071.375</v>
       </c>
       <c r="D47" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E47" t="n">
-        <v>2</v>
+        <v>2.848990227837606</v>
       </c>
       <c r="F47" t="n">
-        <v>2.114764389726374</v>
+        <v>2.89291995286294</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -1853,29 +1853,29 @@
         </is>
       </c>
       <c r="H47" t="n">
-        <v>1.000081729568714</v>
+        <v>1.000000054774468</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>DO_2_4</t>
+          <t>ORP_1_1</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>46103.70833333334</v>
+        <v>46072.875</v>
       </c>
       <c r="C48" s="2" t="n">
-        <v>46104.08333333334</v>
+        <v>46073.08333333334</v>
       </c>
       <c r="D48" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E48" t="n">
-        <v>2.677584717833867</v>
+        <v>2.657825556091456</v>
       </c>
       <c r="F48" t="n">
-        <v>2.780025940040364</v>
+        <v>2.816614046922334</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -1883,7 +1883,7 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>1.000844426489696</v>
+        <v>1.000210598230002</v>
       </c>
     </row>
     <row r="49">
@@ -1893,19 +1893,19 @@
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>45920.16666666666</v>
+        <v>46078.33333333334</v>
       </c>
       <c r="C49" s="2" t="n">
-        <v>45920.375</v>
+        <v>46078.625</v>
       </c>
       <c r="D49" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E49" t="n">
-        <v>2.757376328495986</v>
+        <v>2.746832855958405</v>
       </c>
       <c r="F49" t="n">
-        <v>2.879726012342237</v>
+        <v>2.824440399192632</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -1913,7 +1913,7 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>1.000007312976706</v>
+        <v>1.001550894467055</v>
       </c>
     </row>
     <row r="50">
@@ -1923,19 +1923,19 @@
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>45972.875</v>
+        <v>46094.375</v>
       </c>
       <c r="C50" s="2" t="n">
-        <v>45973.125</v>
+        <v>46094.58333333334</v>
       </c>
       <c r="D50" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E50" t="n">
-        <v>2.809682021993101</v>
+        <v>2.838629155558616</v>
       </c>
       <c r="F50" t="n">
-        <v>2.874583149247187</v>
+        <v>2.891784470303272</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -1943,7 +1943,7 @@
         </is>
       </c>
       <c r="H50" t="n">
-        <v>1.000251210791262</v>
+        <v>1.019566742923476</v>
       </c>
     </row>
     <row r="51">
@@ -1953,19 +1953,19 @@
         </is>
       </c>
       <c r="B51" s="2" t="n">
-        <v>46031.41666666666</v>
+        <v>46103.5</v>
       </c>
       <c r="C51" s="2" t="n">
-        <v>46031.625</v>
+        <v>46103.75</v>
       </c>
       <c r="D51" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E51" t="n">
-        <v>2.834374417406643</v>
+        <v>2.894842078739759</v>
       </c>
       <c r="F51" t="n">
-        <v>2.888146187617946</v>
+        <v>2.932507636981506</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>1.012556226373021</v>
+        <v>1.001234465516338</v>
       </c>
     </row>
     <row r="52">
@@ -1983,19 +1983,19 @@
         </is>
       </c>
       <c r="B52" s="2" t="n">
-        <v>46069.70833333334</v>
+        <v>46114.95833333334</v>
       </c>
       <c r="C52" s="2" t="n">
-        <v>46070.08333333334</v>
+        <v>46115.33333333334</v>
       </c>
       <c r="D52" t="n">
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>2.896610077643929</v>
+        <v>2.798742539278037</v>
       </c>
       <c r="F52" t="n">
-        <v>2.925288845222536</v>
+        <v>2.860378239024466</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -2003,7 +2003,7 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>1.000175276400918</v>
+        <v>1.000170122637875</v>
       </c>
     </row>
     <row r="53">
@@ -2013,19 +2013,19 @@
         </is>
       </c>
       <c r="B53" s="2" t="n">
-        <v>46070.66666666666</v>
+        <v>46115.70833333334</v>
       </c>
       <c r="C53" s="2" t="n">
-        <v>46070.875</v>
+        <v>46115.91666666666</v>
       </c>
       <c r="D53" t="n">
         <v>6</v>
       </c>
       <c r="E53" t="n">
-        <v>2.862447879436455</v>
+        <v>2.82685896567884</v>
       </c>
       <c r="F53" t="n">
-        <v>2.904058513690617</v>
+        <v>2.865204925287654</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -2033,7 +2033,7 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>1.000000824987803</v>
+        <v>1.005129204816508</v>
       </c>
     </row>
     <row r="54">
@@ -2043,19 +2043,19 @@
         </is>
       </c>
       <c r="B54" s="2" t="n">
-        <v>46071.16666666666</v>
+        <v>46117.58333333334</v>
       </c>
       <c r="C54" s="2" t="n">
-        <v>46071.375</v>
+        <v>46117.79166666666</v>
       </c>
       <c r="D54" t="n">
         <v>6</v>
       </c>
       <c r="E54" t="n">
-        <v>2.848990227837606</v>
+        <v>2.722453332391307</v>
       </c>
       <c r="F54" t="n">
-        <v>2.89291995286294</v>
+        <v>2.800563384417298</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -2063,29 +2063,29 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>1.000000054774468</v>
+        <v>1.014371043248799</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>ORP_1_1</t>
+          <t>ORP_1_2</t>
         </is>
       </c>
       <c r="B55" s="2" t="n">
-        <v>46072.875</v>
+        <v>46011.91666666666</v>
       </c>
       <c r="C55" s="2" t="n">
-        <v>46073.08333333334</v>
+        <v>46012.29166666666</v>
       </c>
       <c r="D55" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>2.657825556091456</v>
+        <v>2.757967584852246</v>
       </c>
       <c r="F55" t="n">
-        <v>2.816614046922334</v>
+        <v>2.871753695513218</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -2093,29 +2093,29 @@
         </is>
       </c>
       <c r="H55" t="n">
-        <v>1.000210598230002</v>
+        <v>1.000000448472733</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>ORP_1_1</t>
+          <t>ORP_1_2</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
-        <v>46078.33333333334</v>
+        <v>46013.41666666666</v>
       </c>
       <c r="C56" s="2" t="n">
-        <v>46078.625</v>
+        <v>46013.75</v>
       </c>
       <c r="D56" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E56" t="n">
-        <v>2.746832855958405</v>
+        <v>2.545127570053714</v>
       </c>
       <c r="F56" t="n">
-        <v>2.824440399192632</v>
+        <v>2.771131515972993</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
@@ -2123,29 +2123,29 @@
         </is>
       </c>
       <c r="H56" t="n">
-        <v>1.001550894467055</v>
+        <v>1.000017137212721</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ORP_1_1</t>
+          <t>ORP_1_2</t>
         </is>
       </c>
       <c r="B57" s="2" t="n">
-        <v>46094.375</v>
+        <v>46015.375</v>
       </c>
       <c r="C57" s="2" t="n">
-        <v>46094.58333333334</v>
+        <v>46015.625</v>
       </c>
       <c r="D57" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E57" t="n">
-        <v>2.838629155558616</v>
+        <v>2.691704116627942</v>
       </c>
       <c r="F57" t="n">
-        <v>2.891784470303272</v>
+        <v>2.75093162892788</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -2153,29 +2153,29 @@
         </is>
       </c>
       <c r="H57" t="n">
-        <v>1.019566742923476</v>
+        <v>1.001564884736407</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ORP_1_1</t>
+          <t>ORP_1_2</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
-        <v>46103.5</v>
+        <v>46017.33333333334</v>
       </c>
       <c r="C58" s="2" t="n">
-        <v>46103.75</v>
+        <v>46017.79166666666</v>
       </c>
       <c r="D58" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E58" t="n">
-        <v>2.894842078739759</v>
+        <v>2.387246484347651</v>
       </c>
       <c r="F58" t="n">
-        <v>2.932507636981506</v>
+        <v>2.586018094466748</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -2183,59 +2183,59 @@
         </is>
       </c>
       <c r="H58" t="n">
-        <v>1.001234465516338</v>
+        <v>1.000000351049599</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>ORP_1_1</t>
+          <t>ORP_1_2</t>
         </is>
       </c>
       <c r="B59" s="2" t="n">
-        <v>46114.95833333334</v>
+        <v>46018</v>
       </c>
       <c r="C59" s="2" t="n">
-        <v>46115.33333333334</v>
+        <v>46028.25</v>
       </c>
       <c r="D59" t="n">
-        <v>10</v>
+        <v>247</v>
       </c>
       <c r="E59" t="n">
-        <v>2.798742539278037</v>
+        <v>2.5</v>
       </c>
       <c r="F59" t="n">
-        <v>2.860378239024466</v>
+        <v>2.5</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_regime</t>
         </is>
       </c>
       <c r="H59" t="n">
-        <v>1.000170122637875</v>
+        <v>1.081134041730266</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ORP_1_1</t>
+          <t>ORP_1_2</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
-        <v>46115.70833333334</v>
+        <v>46030.20833333334</v>
       </c>
       <c r="C60" s="2" t="n">
-        <v>46115.91666666666</v>
+        <v>46031.95833333334</v>
       </c>
       <c r="D60" t="n">
-        <v>6</v>
+        <v>43</v>
       </c>
       <c r="E60" t="n">
-        <v>2.82685896567884</v>
+        <v>2.329966376477916</v>
       </c>
       <c r="F60" t="n">
-        <v>2.865204925287654</v>
+        <v>2.487220619812446</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -2243,29 +2243,29 @@
         </is>
       </c>
       <c r="H60" t="n">
-        <v>1.005129204816508</v>
+        <v>1.000390216394669</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>ORP_1_1</t>
+          <t>ORP_1_2</t>
         </is>
       </c>
       <c r="B61" s="2" t="n">
-        <v>46117.58333333334</v>
+        <v>46033.75</v>
       </c>
       <c r="C61" s="2" t="n">
-        <v>46117.79166666666</v>
+        <v>46038.20833333334</v>
       </c>
       <c r="D61" t="n">
-        <v>6</v>
+        <v>108</v>
       </c>
       <c r="E61" t="n">
-        <v>2.722453332391307</v>
+        <v>2.476604834805639</v>
       </c>
       <c r="F61" t="n">
-        <v>2.800563384417298</v>
+        <v>2.499783378100052</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
         </is>
       </c>
       <c r="H61" t="n">
-        <v>1.014371043248799</v>
+        <v>1.100553793654593</v>
       </c>
     </row>
     <row r="62">
@@ -2283,19 +2283,19 @@
         </is>
       </c>
       <c r="B62" s="2" t="n">
-        <v>46011.91666666666</v>
+        <v>46063.875</v>
       </c>
       <c r="C62" s="2" t="n">
-        <v>46012.29166666666</v>
+        <v>46064.08333333334</v>
       </c>
       <c r="D62" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E62" t="n">
-        <v>2.757967584852246</v>
+        <v>2.697827570263692</v>
       </c>
       <c r="F62" t="n">
-        <v>2.871753695513218</v>
+        <v>2.759687927049036</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -2303,7 +2303,7 @@
         </is>
       </c>
       <c r="H62" t="n">
-        <v>1.000000448472733</v>
+        <v>1.000058490844518</v>
       </c>
     </row>
     <row r="63">
@@ -2313,19 +2313,19 @@
         </is>
       </c>
       <c r="B63" s="2" t="n">
-        <v>46013.41666666666</v>
+        <v>46065.83333333334</v>
       </c>
       <c r="C63" s="2" t="n">
-        <v>46013.75</v>
+        <v>46066.25</v>
       </c>
       <c r="D63" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E63" t="n">
-        <v>2.545127570053714</v>
+        <v>2.534839148226271</v>
       </c>
       <c r="F63" t="n">
-        <v>2.771131515972993</v>
+        <v>2.672031339188797</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -2333,7 +2333,7 @@
         </is>
       </c>
       <c r="H63" t="n">
-        <v>1.000017137212721</v>
+        <v>1.000591289877526</v>
       </c>
     </row>
     <row r="64">
@@ -2343,19 +2343,19 @@
         </is>
       </c>
       <c r="B64" s="2" t="n">
-        <v>46015.375</v>
+        <v>46067.29166666666</v>
       </c>
       <c r="C64" s="2" t="n">
-        <v>46015.625</v>
+        <v>46067.58333333334</v>
       </c>
       <c r="D64" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E64" t="n">
-        <v>2.691704116627942</v>
+        <v>2.592961524228548</v>
       </c>
       <c r="F64" t="n">
-        <v>2.75093162892788</v>
+        <v>2.729217713985539</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -2363,7 +2363,7 @@
         </is>
       </c>
       <c r="H64" t="n">
-        <v>1.001564884736407</v>
+        <v>1.000176110832394</v>
       </c>
     </row>
     <row r="65">
@@ -2373,19 +2373,19 @@
         </is>
       </c>
       <c r="B65" s="2" t="n">
-        <v>46017.33333333334</v>
+        <v>46068.33333333334</v>
       </c>
       <c r="C65" s="2" t="n">
-        <v>46017.79166666666</v>
+        <v>46068.625</v>
       </c>
       <c r="D65" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E65" t="n">
-        <v>2.387246484347651</v>
+        <v>2.480221425257873</v>
       </c>
       <c r="F65" t="n">
-        <v>2.586018094466748</v>
+        <v>2.663636670467292</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -2393,7 +2393,7 @@
         </is>
       </c>
       <c r="H65" t="n">
-        <v>1.000000351049599</v>
+        <v>1.001407905053316</v>
       </c>
     </row>
     <row r="66">
@@ -2403,27 +2403,27 @@
         </is>
       </c>
       <c r="B66" s="2" t="n">
-        <v>46018</v>
+        <v>46069.70833333334</v>
       </c>
       <c r="C66" s="2" t="n">
-        <v>46028.25</v>
+        <v>46077.91666666666</v>
       </c>
       <c r="D66" t="n">
-        <v>247</v>
+        <v>198</v>
       </c>
       <c r="E66" t="n">
-        <v>2.5</v>
+        <v>2.413148214499939</v>
       </c>
       <c r="F66" t="n">
-        <v>2.5</v>
+        <v>2.501817813877794</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Q_regime</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H66" t="n">
-        <v>1.081134041730266</v>
+        <v>1.000000021182844</v>
       </c>
     </row>
     <row r="67">
@@ -2433,19 +2433,19 @@
         </is>
       </c>
       <c r="B67" s="2" t="n">
-        <v>46030.20833333334</v>
+        <v>46078.41666666666</v>
       </c>
       <c r="C67" s="2" t="n">
-        <v>46031.95833333334</v>
+        <v>46082.125</v>
       </c>
       <c r="D67" t="n">
-        <v>43</v>
+        <v>90</v>
       </c>
       <c r="E67" t="n">
-        <v>2.329966376477916</v>
+        <v>2.5</v>
       </c>
       <c r="F67" t="n">
-        <v>2.487220619812446</v>
+        <v>2.5</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
@@ -2453,7 +2453,7 @@
         </is>
       </c>
       <c r="H67" t="n">
-        <v>1.000390216394669</v>
+        <v>1.068234383831886</v>
       </c>
     </row>
     <row r="68">
@@ -2463,27 +2463,27 @@
         </is>
       </c>
       <c r="B68" s="2" t="n">
-        <v>46033.75</v>
+        <v>46082.25</v>
       </c>
       <c r="C68" s="2" t="n">
-        <v>46038.20833333334</v>
+        <v>46089.25</v>
       </c>
       <c r="D68" t="n">
-        <v>108</v>
+        <v>169</v>
       </c>
       <c r="E68" t="n">
-        <v>2.476604834805639</v>
+        <v>2.5</v>
       </c>
       <c r="F68" t="n">
-        <v>2.499783378100052</v>
+        <v>2.5</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_regime</t>
         </is>
       </c>
       <c r="H68" t="n">
-        <v>1.100553793654593</v>
+        <v>1.333577532071762</v>
       </c>
     </row>
     <row r="69">
@@ -2493,19 +2493,19 @@
         </is>
       </c>
       <c r="B69" s="2" t="n">
-        <v>46063.875</v>
+        <v>46115</v>
       </c>
       <c r="C69" s="2" t="n">
-        <v>46064.08333333334</v>
+        <v>46115.29166666666</v>
       </c>
       <c r="D69" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E69" t="n">
-        <v>2.697827570263692</v>
+        <v>2.481712743778947</v>
       </c>
       <c r="F69" t="n">
-        <v>2.759687927049036</v>
+        <v>2.645869648668306</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="H69" t="n">
-        <v>1.000058490844518</v>
+        <v>1.102732574463459</v>
       </c>
     </row>
     <row r="70">
@@ -2523,19 +2523,19 @@
         </is>
       </c>
       <c r="B70" s="2" t="n">
-        <v>46065.83333333334</v>
+        <v>46117.58333333334</v>
       </c>
       <c r="C70" s="2" t="n">
-        <v>46066.25</v>
+        <v>46117.95833333334</v>
       </c>
       <c r="D70" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>2.534839148226271</v>
+        <v>2.5</v>
       </c>
       <c r="F70" t="n">
-        <v>2.672031339188797</v>
+        <v>2.620961897829237</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
@@ -2543,7 +2543,7 @@
         </is>
       </c>
       <c r="H70" t="n">
-        <v>1.000591289877526</v>
+        <v>1.546691130829444</v>
       </c>
     </row>
     <row r="71">
@@ -2553,19 +2553,19 @@
         </is>
       </c>
       <c r="B71" s="2" t="n">
-        <v>46067.29166666666</v>
+        <v>46118.5</v>
       </c>
       <c r="C71" s="2" t="n">
-        <v>46067.58333333334</v>
+        <v>46122.45833333334</v>
       </c>
       <c r="D71" t="n">
-        <v>8</v>
+        <v>96</v>
       </c>
       <c r="E71" t="n">
-        <v>2.592961524228548</v>
+        <v>2.426672063099368</v>
       </c>
       <c r="F71" t="n">
-        <v>2.729217713985539</v>
+        <v>2.498788344672366</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
@@ -2573,83 +2573,83 @@
         </is>
       </c>
       <c r="H71" t="n">
-        <v>1.000176110832394</v>
+        <v>1.016919746167972</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>ORP_1_2</t>
+          <t>ORP_1_3</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
-        <v>46068.33333333334</v>
+        <v>45944.5</v>
       </c>
       <c r="C72" s="2" t="n">
-        <v>46068.625</v>
+        <v>45944.70833333334</v>
       </c>
       <c r="D72" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E72" t="n">
-        <v>2.480221425257873</v>
+        <v>2.359579249772268</v>
       </c>
       <c r="F72" t="n">
-        <v>2.663636670467292</v>
+        <v>2.540101005989568</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_step</t>
         </is>
       </c>
       <c r="H72" t="n">
-        <v>1.001407905053316</v>
+        <v>1.239094636012759</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>ORP_1_2</t>
+          <t>ORP_1_3</t>
         </is>
       </c>
       <c r="B73" s="2" t="n">
-        <v>46069.70833333334</v>
+        <v>45945.25</v>
       </c>
       <c r="C73" s="2" t="n">
-        <v>46077.91666666666</v>
+        <v>45945.45833333334</v>
       </c>
       <c r="D73" t="n">
-        <v>198</v>
+        <v>6</v>
       </c>
       <c r="E73" t="n">
-        <v>2.413148214499939</v>
+        <v>2.5</v>
       </c>
       <c r="F73" t="n">
-        <v>2.501817813877794</v>
+        <v>2.5</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_regime</t>
         </is>
       </c>
       <c r="H73" t="n">
-        <v>1.000000021182844</v>
+        <v>1.961678843667339</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>ORP_1_2</t>
+          <t>ORP_1_3</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
-        <v>46078.41666666666</v>
+        <v>45946.5</v>
       </c>
       <c r="C74" s="2" t="n">
-        <v>46082.125</v>
+        <v>45948.41666666666</v>
       </c>
       <c r="D74" t="n">
-        <v>90</v>
+        <v>47</v>
       </c>
       <c r="E74" t="n">
         <v>2.5</v>
@@ -2659,27 +2659,27 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_regime</t>
         </is>
       </c>
       <c r="H74" t="n">
-        <v>1.068234383831886</v>
+        <v>2.108098132368428</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>ORP_1_2</t>
+          <t>ORP_1_3</t>
         </is>
       </c>
       <c r="B75" s="2" t="n">
-        <v>46082.25</v>
+        <v>45948.58333333334</v>
       </c>
       <c r="C75" s="2" t="n">
-        <v>46089.25</v>
+        <v>45949.5</v>
       </c>
       <c r="D75" t="n">
-        <v>169</v>
+        <v>23</v>
       </c>
       <c r="E75" t="n">
         <v>2.5</v>
@@ -2689,63 +2689,63 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Q_regime</t>
+          <t>Q_step</t>
         </is>
       </c>
       <c r="H75" t="n">
-        <v>1.333577532071762</v>
+        <v>3.133136153004526</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>ORP_1_2</t>
+          <t>ORP_1_3</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
-        <v>46115</v>
+        <v>45985.875</v>
       </c>
       <c r="C76" s="2" t="n">
-        <v>46115.29166666666</v>
+        <v>45986.08333333334</v>
       </c>
       <c r="D76" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E76" t="n">
-        <v>2.481712743778947</v>
+        <v>2.532284377008832</v>
       </c>
       <c r="F76" t="n">
-        <v>2.645869648668306</v>
+        <v>2.702907353326314</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_step</t>
         </is>
       </c>
       <c r="H76" t="n">
-        <v>1.102732574463459</v>
+        <v>1.156662891187058</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>ORP_1_2</t>
+          <t>ORP_2_1</t>
         </is>
       </c>
       <c r="B77" s="2" t="n">
-        <v>46117.58333333334</v>
+        <v>45912.66666666666</v>
       </c>
       <c r="C77" s="2" t="n">
-        <v>46117.95833333334</v>
+        <v>45912.91666666666</v>
       </c>
       <c r="D77" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E77" t="n">
-        <v>2.5</v>
+        <v>2.916749424863698</v>
       </c>
       <c r="F77" t="n">
-        <v>2.620961897829237</v>
+        <v>2.958434285225183</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -2753,29 +2753,29 @@
         </is>
       </c>
       <c r="H77" t="n">
-        <v>1.546691130829444</v>
+        <v>1.000403757743586</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>ORP_1_2</t>
+          <t>ORP_2_1</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
-        <v>46118.5</v>
+        <v>45913.58333333334</v>
       </c>
       <c r="C78" s="2" t="n">
-        <v>46122.45833333334</v>
+        <v>45914</v>
       </c>
       <c r="D78" t="n">
-        <v>96</v>
+        <v>11</v>
       </c>
       <c r="E78" t="n">
-        <v>2.426672063099368</v>
+        <v>2.813665244581917</v>
       </c>
       <c r="F78" t="n">
-        <v>2.498788344672366</v>
+        <v>2.870842326941625</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -2783,53 +2783,53 @@
         </is>
       </c>
       <c r="H78" t="n">
-        <v>1.016919746167972</v>
+        <v>1.001934196184946</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>ORP_1_3</t>
+          <t>ORP_2_2</t>
         </is>
       </c>
       <c r="B79" s="2" t="n">
-        <v>45944.5</v>
+        <v>46018.75</v>
       </c>
       <c r="C79" s="2" t="n">
-        <v>45944.70833333334</v>
+        <v>46019</v>
       </c>
       <c r="D79" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E79" t="n">
-        <v>2.359579249772268</v>
+        <v>2.734094841154886</v>
       </c>
       <c r="F79" t="n">
-        <v>2.540101005989568</v>
+        <v>2.860673160381919</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Q_step</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H79" t="n">
-        <v>1.239094636012759</v>
+        <v>1.031984641824361</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>ORP_1_3</t>
+          <t>ORP_2_2</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
-        <v>45945.25</v>
+        <v>46036.75</v>
       </c>
       <c r="C80" s="2" t="n">
-        <v>45945.45833333334</v>
+        <v>46037.45833333334</v>
       </c>
       <c r="D80" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="E80" t="n">
         <v>2.5</v>
@@ -2843,53 +2843,53 @@
         </is>
       </c>
       <c r="H80" t="n">
-        <v>1.961678843667339</v>
+        <v>1.922445730625928</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>ORP_1_3</t>
+          <t>ORP_2_2</t>
         </is>
       </c>
       <c r="B81" s="2" t="n">
-        <v>45946.5</v>
+        <v>46080.58333333334</v>
       </c>
       <c r="C81" s="2" t="n">
-        <v>45948.41666666666</v>
+        <v>46080.79166666666</v>
       </c>
       <c r="D81" t="n">
-        <v>47</v>
+        <v>6</v>
       </c>
       <c r="E81" t="n">
-        <v>2.5</v>
+        <v>2.81960042268659</v>
       </c>
       <c r="F81" t="n">
-        <v>2.5</v>
+        <v>2.893198009776475</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Q_regime</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H81" t="n">
-        <v>2.108098132368428</v>
+        <v>1.005173111560453</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>ORP_1_3</t>
+          <t>ORP_2_2</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
-        <v>45948.58333333334</v>
+        <v>46119</v>
       </c>
       <c r="C82" s="2" t="n">
-        <v>45949.5</v>
+        <v>46122.45833333334</v>
       </c>
       <c r="D82" t="n">
-        <v>23</v>
+        <v>84</v>
       </c>
       <c r="E82" t="n">
         <v>2.5</v>
@@ -2899,220 +2899,10 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Q_step</t>
+          <t>Q_regime</t>
         </is>
       </c>
       <c r="H82" t="n">
-        <v>3.133136153004526</v>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>ORP_1_3</t>
-        </is>
-      </c>
-      <c r="B83" s="2" t="n">
-        <v>45985.875</v>
-      </c>
-      <c r="C83" s="2" t="n">
-        <v>45986.08333333334</v>
-      </c>
-      <c r="D83" t="n">
-        <v>6</v>
-      </c>
-      <c r="E83" t="n">
-        <v>2.532284377008832</v>
-      </c>
-      <c r="F83" t="n">
-        <v>2.702907353326314</v>
-      </c>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>Q_step</t>
-        </is>
-      </c>
-      <c r="H83" t="n">
-        <v>1.156662891187058</v>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>ORP_2_1</t>
-        </is>
-      </c>
-      <c r="B84" s="2" t="n">
-        <v>45912.66666666666</v>
-      </c>
-      <c r="C84" s="2" t="n">
-        <v>45912.91666666666</v>
-      </c>
-      <c r="D84" t="n">
-        <v>7</v>
-      </c>
-      <c r="E84" t="n">
-        <v>2.916749424863698</v>
-      </c>
-      <c r="F84" t="n">
-        <v>2.958434285225183</v>
-      </c>
-      <c r="G84" t="inlineStr">
-        <is>
-          <t>Q_drift</t>
-        </is>
-      </c>
-      <c r="H84" t="n">
-        <v>1.000403757743586</v>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>ORP_2_1</t>
-        </is>
-      </c>
-      <c r="B85" s="2" t="n">
-        <v>45913.58333333334</v>
-      </c>
-      <c r="C85" s="2" t="n">
-        <v>45914</v>
-      </c>
-      <c r="D85" t="n">
-        <v>11</v>
-      </c>
-      <c r="E85" t="n">
-        <v>2.813665244581917</v>
-      </c>
-      <c r="F85" t="n">
-        <v>2.870842326941625</v>
-      </c>
-      <c r="G85" t="inlineStr">
-        <is>
-          <t>Q_drift</t>
-        </is>
-      </c>
-      <c r="H85" t="n">
-        <v>1.001934196184946</v>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>ORP_2_2</t>
-        </is>
-      </c>
-      <c r="B86" s="2" t="n">
-        <v>46018.75</v>
-      </c>
-      <c r="C86" s="2" t="n">
-        <v>46019</v>
-      </c>
-      <c r="D86" t="n">
-        <v>7</v>
-      </c>
-      <c r="E86" t="n">
-        <v>2.734094841154886</v>
-      </c>
-      <c r="F86" t="n">
-        <v>2.860673160381919</v>
-      </c>
-      <c r="G86" t="inlineStr">
-        <is>
-          <t>Q_drift</t>
-        </is>
-      </c>
-      <c r="H86" t="n">
-        <v>1.031984641824361</v>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>ORP_2_2</t>
-        </is>
-      </c>
-      <c r="B87" s="2" t="n">
-        <v>46036.75</v>
-      </c>
-      <c r="C87" s="2" t="n">
-        <v>46037.45833333334</v>
-      </c>
-      <c r="D87" t="n">
-        <v>18</v>
-      </c>
-      <c r="E87" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="F87" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="G87" t="inlineStr">
-        <is>
-          <t>Q_regime</t>
-        </is>
-      </c>
-      <c r="H87" t="n">
-        <v>1.922445730625928</v>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>ORP_2_2</t>
-        </is>
-      </c>
-      <c r="B88" s="2" t="n">
-        <v>46080.58333333334</v>
-      </c>
-      <c r="C88" s="2" t="n">
-        <v>46080.79166666666</v>
-      </c>
-      <c r="D88" t="n">
-        <v>6</v>
-      </c>
-      <c r="E88" t="n">
-        <v>2.81960042268659</v>
-      </c>
-      <c r="F88" t="n">
-        <v>2.893198009776475</v>
-      </c>
-      <c r="G88" t="inlineStr">
-        <is>
-          <t>Q_drift</t>
-        </is>
-      </c>
-      <c r="H88" t="n">
-        <v>1.005173111560453</v>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>ORP_2_2</t>
-        </is>
-      </c>
-      <c r="B89" s="2" t="n">
-        <v>46119</v>
-      </c>
-      <c r="C89" s="2" t="n">
-        <v>46122.45833333334</v>
-      </c>
-      <c r="D89" t="n">
-        <v>84</v>
-      </c>
-      <c r="E89" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="F89" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="G89" t="inlineStr">
-        <is>
-          <t>Q_regime</t>
-        </is>
-      </c>
-      <c r="H89" t="n">
         <v>1.160462951377068</v>
       </c>
     </row>
@@ -3599,19 +3389,19 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>45923.29166666666</v>
+        <v>45914.25</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>45927.20833333334</v>
+        <v>45923.08333333334</v>
       </c>
       <c r="D16" t="n">
-        <v>95</v>
+        <v>213</v>
       </c>
       <c r="E16" t="n">
         <v>2.5</v>
       </c>
       <c r="F16" t="n">
-        <v>2.504750233674428</v>
+        <v>2.5</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -3619,7 +3409,7 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>1.007870807954773</v>
+        <v>1.000027425415349</v>
       </c>
     </row>
     <row r="17">
@@ -3629,13 +3419,13 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>45914.25</v>
+        <v>45931.375</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>45923.08333333334</v>
+        <v>45939.25</v>
       </c>
       <c r="D17" t="n">
-        <v>213</v>
+        <v>190</v>
       </c>
       <c r="E17" t="n">
         <v>2.5</v>
@@ -3649,7 +3439,7 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>1.000027425415349</v>
+        <v>1.000000013028375</v>
       </c>
     </row>
     <row r="18">
@@ -3659,19 +3449,19 @@
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>45927.29166666666</v>
+        <v>45929.29166666666</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>45929.08333333334</v>
+        <v>45931.20833333334</v>
       </c>
       <c r="D18" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="E18" t="n">
         <v>2.5</v>
       </c>
       <c r="F18" t="n">
-        <v>2.513093523236048</v>
+        <v>2.516133291750057</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -3679,7 +3469,7 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>1.000024569032804</v>
+        <v>1.005320194675679</v>
       </c>
     </row>
     <row r="19">
@@ -3689,19 +3479,19 @@
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>45931.375</v>
+        <v>45927.29166666666</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>45939.25</v>
+        <v>45929.08333333334</v>
       </c>
       <c r="D19" t="n">
-        <v>190</v>
+        <v>44</v>
       </c>
       <c r="E19" t="n">
         <v>2.5</v>
       </c>
       <c r="F19" t="n">
-        <v>2.5</v>
+        <v>2.513093523236048</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -3709,7 +3499,7 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>1.000000013028375</v>
+        <v>1.000024569032804</v>
       </c>
     </row>
     <row r="20">
@@ -3719,19 +3509,19 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>45929.29166666666</v>
+        <v>45923.29166666666</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>45931.20833333334</v>
+        <v>45927.20833333334</v>
       </c>
       <c r="D20" t="n">
-        <v>47</v>
+        <v>95</v>
       </c>
       <c r="E20" t="n">
         <v>2.5</v>
       </c>
       <c r="F20" t="n">
-        <v>2.516133291750057</v>
+        <v>2.504750233674428</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -3739,7 +3529,7 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>1.005320194675679</v>
+        <v>1.007870807954773</v>
       </c>
     </row>
     <row r="21">
@@ -3791,7 +3581,7 @@
         <v>2</v>
       </c>
       <c r="F22" t="n">
-        <v>2.114764389726374</v>
+        <v>2.117137735246667</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -3799,7 +3589,7 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>1.000081729568714</v>
+        <v>1.011071265909375</v>
       </c>
     </row>
     <row r="23">
@@ -3809,19 +3599,19 @@
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>45998.66666666666</v>
+        <v>46011.91666666666</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>45998.875</v>
+        <v>46012.16666666666</v>
       </c>
       <c r="D23" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E23" t="n">
-        <v>2.211936251292717</v>
+        <v>2.396590681906827</v>
       </c>
       <c r="F23" t="n">
-        <v>2.479658830044532</v>
+        <v>2.583110821007263</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -3829,7 +3619,7 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>1.0189217456638</v>
+        <v>1.000022499433851</v>
       </c>
     </row>
     <row r="24">
@@ -3839,19 +3629,19 @@
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>46011.91666666666</v>
+        <v>45984.45833333334</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>46012.20833333334</v>
+        <v>45984.91666666666</v>
       </c>
       <c r="D24" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E24" t="n">
-        <v>2.392805004675806</v>
+        <v>2.44799296816425</v>
       </c>
       <c r="F24" t="n">
-        <v>2.596736357047955</v>
+        <v>2.717725229822283</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -3859,7 +3649,7 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>1.000015078979207</v>
+        <v>1.000001210556082</v>
       </c>
     </row>
     <row r="25">
@@ -3869,19 +3659,19 @@
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>45984.45833333334</v>
+        <v>46013.66666666666</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>45984.91666666666</v>
+        <v>46014.16666666666</v>
       </c>
       <c r="D25" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E25" t="n">
-        <v>2.447935866890584</v>
+        <v>2.451283473014483</v>
       </c>
       <c r="F25" t="n">
-        <v>2.718102655457825</v>
+        <v>2.664910159560438</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -3889,7 +3679,7 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>1.000001103825005</v>
+        <v>1.000000001127826</v>
       </c>
     </row>
     <row r="26">
@@ -3899,27 +3689,27 @@
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>46013.66666666666</v>
+        <v>45985</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>46014.16666666666</v>
+        <v>45985.54166666666</v>
       </c>
       <c r="D26" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E26" t="n">
-        <v>2.451277291557278</v>
+        <v>2.550175579847397</v>
       </c>
       <c r="F26" t="n">
-        <v>2.664274531537799</v>
+        <v>2.71946138852274</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_step</t>
         </is>
       </c>
       <c r="H26" t="n">
-        <v>1.000000000141117</v>
+        <v>1.156662891187058</v>
       </c>
     </row>
     <row r="27">
@@ -3929,19 +3719,19 @@
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>46068.75</v>
+        <v>46011.5</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>46069.125</v>
+        <v>46011.83333333334</v>
       </c>
       <c r="D27" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E27" t="n">
-        <v>2.534498966663721</v>
+        <v>2.567221759903792</v>
       </c>
       <c r="F27" t="n">
-        <v>2.670607565166778</v>
+        <v>2.641917370543523</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -3949,7 +3739,7 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>1.029970506055951</v>
+        <v>1.000000061891391</v>
       </c>
     </row>
     <row r="28">
@@ -3959,27 +3749,27 @@
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>45985</v>
+        <v>45982.66666666666</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>45985.54166666666</v>
+        <v>45983.41666666666</v>
       </c>
       <c r="D28" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="E28" t="n">
-        <v>2.550175579847397</v>
+        <v>2.593419013399966</v>
       </c>
       <c r="F28" t="n">
-        <v>2.71946138852274</v>
+        <v>2.829096550849842</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Q_step</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H28" t="n">
-        <v>1.156662891187058</v>
+        <v>1.000004287752132</v>
       </c>
     </row>
     <row r="29">
@@ -3989,19 +3779,19 @@
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>46029.625</v>
+        <v>45920.75</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>46029.875</v>
+        <v>45921</v>
       </c>
       <c r="D29" t="n">
         <v>7</v>
       </c>
       <c r="E29" t="n">
-        <v>2.567062194481823</v>
+        <v>2.645057429847372</v>
       </c>
       <c r="F29" t="n">
-        <v>2.755760587104711</v>
+        <v>2.860199471141084</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -4009,7 +3799,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>1.001531969385012</v>
+        <v>1.008206399446979</v>
       </c>
     </row>
     <row r="30">
@@ -4019,19 +3809,19 @@
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>46011.5</v>
+        <v>46029.66666666666</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>46011.83333333334</v>
+        <v>46029.875</v>
       </c>
       <c r="D30" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E30" t="n">
-        <v>2.567194367272065</v>
+        <v>2.650301756052542</v>
       </c>
       <c r="F30" t="n">
-        <v>2.64530938286319</v>
+        <v>2.783738827060561</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -4039,7 +3829,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>1.000000067627254</v>
+        <v>1.003314581123384</v>
       </c>
     </row>
     <row r="31">
@@ -4049,19 +3839,19 @@
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>46077.70833333334</v>
+        <v>46103.75</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>46078</v>
+        <v>46104.08333333334</v>
       </c>
       <c r="D31" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E31" t="n">
-        <v>2.588607853112589</v>
+        <v>2.701271638760034</v>
       </c>
       <c r="F31" t="n">
-        <v>2.84003479810486</v>
+        <v>2.829865795819057</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -4069,7 +3859,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>1.03956381193685</v>
+        <v>1.027031614956905</v>
       </c>
     </row>
     <row r="32">
@@ -4589,13 +4379,13 @@
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>46018</v>
+        <v>46082.25</v>
       </c>
       <c r="C49" s="2" t="n">
-        <v>46028.25</v>
+        <v>46089.25</v>
       </c>
       <c r="D49" t="n">
-        <v>247</v>
+        <v>169</v>
       </c>
       <c r="E49" t="n">
         <v>2.5</v>
@@ -4609,7 +4399,7 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>1.081134041730266</v>
+        <v>1.333577532071762</v>
       </c>
     </row>
     <row r="50">
@@ -4619,13 +4409,13 @@
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>46078.41666666666</v>
+        <v>46018</v>
       </c>
       <c r="C50" s="2" t="n">
-        <v>46082.125</v>
+        <v>46028.25</v>
       </c>
       <c r="D50" t="n">
-        <v>90</v>
+        <v>247</v>
       </c>
       <c r="E50" t="n">
         <v>2.5</v>
@@ -4635,11 +4425,11 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_regime</t>
         </is>
       </c>
       <c r="H50" t="n">
-        <v>1.068234383831886</v>
+        <v>1.081134041730266</v>
       </c>
     </row>
     <row r="51">
@@ -4649,13 +4439,13 @@
         </is>
       </c>
       <c r="B51" s="2" t="n">
-        <v>46082.25</v>
+        <v>46078.41666666666</v>
       </c>
       <c r="C51" s="2" t="n">
-        <v>46089.25</v>
+        <v>46082.125</v>
       </c>
       <c r="D51" t="n">
-        <v>169</v>
+        <v>90</v>
       </c>
       <c r="E51" t="n">
         <v>2.5</v>
@@ -4665,11 +4455,11 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Q_regime</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="H51" t="n">
-        <v>1.333577532071762</v>
+        <v>1.068234383831886</v>
       </c>
     </row>
     <row r="52">
@@ -4709,13 +4499,13 @@
         </is>
       </c>
       <c r="B53" s="2" t="n">
-        <v>45948.58333333334</v>
+        <v>45945.25</v>
       </c>
       <c r="C53" s="2" t="n">
-        <v>45949.5</v>
+        <v>45945.45833333334</v>
       </c>
       <c r="D53" t="n">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="E53" t="n">
         <v>2.5</v>
@@ -4725,11 +4515,11 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Q_step</t>
+          <t>Q_regime</t>
         </is>
       </c>
       <c r="H53" t="n">
-        <v>3.133136153004526</v>
+        <v>1.961678843667339</v>
       </c>
     </row>
     <row r="54">
@@ -4769,13 +4559,13 @@
         </is>
       </c>
       <c r="B55" s="2" t="n">
-        <v>45945.25</v>
+        <v>45948.58333333334</v>
       </c>
       <c r="C55" s="2" t="n">
-        <v>45945.45833333334</v>
+        <v>45949.5</v>
       </c>
       <c r="D55" t="n">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="E55" t="n">
         <v>2.5</v>
@@ -4785,11 +4575,11 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Q_regime</t>
+          <t>Q_step</t>
         </is>
       </c>
       <c r="H55" t="n">
-        <v>1.961678843667339</v>
+        <v>3.133136153004526</v>
       </c>
     </row>
     <row r="56">
@@ -5013,7 +4803,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5244,13 +5034,13 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="D11" t="n">
-        <v>159</v>
+        <v>108</v>
       </c>
       <c r="E11" t="n">
-        <v>2.560832894283463</v>
+        <v>2.544905785287976</v>
       </c>
     </row>
     <row r="12">
@@ -5261,44 +5051,44 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Q_spike</t>
+          <t>Q_step</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D12" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="E12" t="n">
-        <v>2.682590823715822</v>
+        <v>2.663451209623768</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>DO_2_4</t>
+          <t>ORP_1_1</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Q_step</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="D13" t="n">
-        <v>20</v>
+        <v>90</v>
       </c>
       <c r="E13" t="n">
-        <v>2.663451209623768</v>
+        <v>2.807358879731549</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ORP_1_1</t>
+          <t>ORP_1_2</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -5307,13 +5097,13 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D14" t="n">
-        <v>90</v>
+        <v>624</v>
       </c>
       <c r="E14" t="n">
-        <v>2.807358879731549</v>
+        <v>2.521066643767983</v>
       </c>
     </row>
     <row r="15">
@@ -5324,23 +5114,23 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_regime</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="D15" t="n">
-        <v>624</v>
+        <v>416</v>
       </c>
       <c r="E15" t="n">
-        <v>2.521066643767983</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ORP_1_2</t>
+          <t>ORP_1_3</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -5352,7 +5142,7 @@
         <v>2</v>
       </c>
       <c r="D16" t="n">
-        <v>416</v>
+        <v>53</v>
       </c>
       <c r="E16" t="n">
         <v>2.5</v>
@@ -5366,44 +5156,44 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Q_regime</t>
+          <t>Q_step</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D17" t="n">
-        <v>53</v>
+        <v>35</v>
       </c>
       <c r="E17" t="n">
-        <v>2.5</v>
+        <v>2.463954542260367</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ORP_1_3</t>
+          <t>ORP_2_1</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Q_step</t>
+          <t>Q_drift</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D18" t="n">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="E18" t="n">
-        <v>2.463954542260367</v>
+        <v>2.865207334722808</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ORP_2_1</t>
+          <t>ORP_2_2</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -5415,10 +5205,10 @@
         <v>2</v>
       </c>
       <c r="D19" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E19" t="n">
-        <v>2.865207334722808</v>
+        <v>2.776847631920738</v>
       </c>
     </row>
     <row r="20">
@@ -5429,37 +5219,16 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Q_drift</t>
+          <t>Q_regime</t>
         </is>
       </c>
       <c r="C20" t="n">
         <v>2</v>
       </c>
       <c r="D20" t="n">
-        <v>13</v>
+        <v>102</v>
       </c>
       <c r="E20" t="n">
-        <v>2.776847631920738</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>ORP_2_2</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Q_regime</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>2</v>
-      </c>
-      <c r="D21" t="n">
-        <v>102</v>
-      </c>
-      <c r="E21" t="n">
         <v>2.5</v>
       </c>
     </row>

</xml_diff>